<commit_message>
T-0559: two readings of printed pages 229 and 231, settled against the sheets
The two readings differ on ONE cell per page, not 20 and 25 — those figures
compared each reading through its own committed-column mask. All six disputed
footings re-read at 4x-12x; page 229 column 1 de-committed, column 14 committed.
</commit_message>
<xml_diff>
--- a/chicago/reference/census1840/validation/T-0504_1840_name_serial_crosswalk.xlsx
+++ b/chicago/reference/census1840/validation/T-0504_1840_name_serial_crosswalk.xlsx
@@ -1395,14 +1395,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>5101709</t>
-        </is>
-      </c>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J16" t="n">
@@ -1413,7 +1409,7 @@
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>contested: serial 5101709 is the sole fingerprint match for 2 different lines (33S7-9YYJ-2T line 15, 33S7-9YYJ-9M5 line 22), and a serial may not be attached twice, so none of them keeps it</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -11566,7 +11562,7 @@
       <c r="H188" t="inlineStr"/>
       <c r="I188" t="inlineStr">
         <is>
-          <t>ambiguous(14)</t>
+          <t>ambiguous(8)</t>
         </is>
       </c>
       <c r="J188" t="n">
@@ -11574,14 +11570,14 @@
       </c>
       <c r="K188" t="inlineStr">
         <is>
-          <t>5101354;5101370;5101379;5101712;5101732;5101757;5101821;5101896;5101924;5101941;5102016;5102149;5102154;5102164</t>
+          <t>5101712;5101821;5101896;5101924;5101941;5102149;5102154;5102164</t>
         </is>
       </c>
       <c r="L188" t="inlineStr"/>
       <c r="M188" t="inlineStr"/>
       <c r="N188" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 14 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 8 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O188" t="inlineStr">
@@ -11625,7 +11621,7 @@
       <c r="H189" t="inlineStr"/>
       <c r="I189" t="inlineStr">
         <is>
-          <t>ambiguous(24)</t>
+          <t>ambiguous(29)</t>
         </is>
       </c>
       <c r="J189" t="n">
@@ -11633,14 +11629,14 @@
       </c>
       <c r="K189" t="inlineStr">
         <is>
-          <t>5101307;5101362;5101440;5101450;5101509;5101516;5101580;5101628;5101650;5101654;5101655;5101728;5101776;5101783;5101852;5101857;5101944;5101969;5101976;5102005;5102045;5102094;5102137;5102157</t>
+          <t>5101254;5101263;5101344;5101362;5101450;5101478;5101509;5101516;5101561;5101580;5101628;5101650;5101654;5101655;5101691;5101735;5101776;5101783;5101800;5101805;5101857;5101871;5101878;5101881;5101969;5102045;5102108;5102148;5102160</t>
         </is>
       </c>
       <c r="L189" t="inlineStr"/>
       <c r="M189" t="inlineStr"/>
       <c r="N189" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 24 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 29 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O189" t="inlineStr">
@@ -11681,14 +11677,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H190" t="inlineStr">
-        <is>
-          <t>5101945</t>
-        </is>
-      </c>
+      <c r="H190" t="inlineStr"/>
       <c r="I190" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J190" t="n">
@@ -11699,7 +11691,7 @@
       <c r="M190" t="inlineStr"/>
       <c r="N190" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O190" t="inlineStr">
@@ -11743,7 +11735,7 @@
       <c r="H191" t="inlineStr"/>
       <c r="I191" t="inlineStr">
         <is>
-          <t>ambiguous(33)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J191" t="n">
@@ -11751,22 +11743,14 @@
       </c>
       <c r="K191" t="inlineStr">
         <is>
-          <t>5101309;5101427;5101502;5101537;5101555;5101557;5101583;5101648;5101653;5101682;5101702;5101722;5101813;5101827;5101864;5101869;5101890;5101895;5101905;5101909;5101937;5101939;5101946;5101973;5102000;5102011;5102038;5102044;5102052;5102105;5102109;5102144;5102187</t>
-        </is>
-      </c>
-      <c r="L191" t="inlineStr">
-        <is>
-          <t>5101946</t>
-        </is>
-      </c>
-      <c r="M191" t="inlineStr">
-        <is>
-          <t>lines 3 and 6 resolve uniquely to serials 5101945 and 5101948; of this line's 33 candidates exactly one, 5101946, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
+        </is>
+      </c>
+      <c r="L191" t="inlineStr"/>
+      <c r="M191" t="inlineStr"/>
       <c r="N191" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 33 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O191" t="inlineStr">
@@ -11810,7 +11794,7 @@
       <c r="H192" t="inlineStr"/>
       <c r="I192" t="inlineStr">
         <is>
-          <t>ambiguous(80)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J192" t="n">
@@ -11818,22 +11802,14 @@
       </c>
       <c r="K192" t="inlineStr">
         <is>
-          <t>5101273;5101279;5101291;5101294;5101321;5101324;5101337;5101385;5101432;5101434;5101443;5101464;5101465;5101476;5101479;5101485;5101540;5101551;5101552;5101589;5101606;5101609;5101631;5101656;5101663;5101669;5101678;5101684;5101685;5101689;5101708;5101710;5101723;5101726;5101739;5101743;5101744;5101759;5101764;5101765;5101779;5101780;5101784;5101792;5101794;5101807;5101808;5101812;5101820;5101822;5101842;5101853;5101873;5101880;5101882;5101883;5101898;5101906;5101918;5101928;5101935;5101947;5101954;5101956;5101980;5101985;5101986;5101990;5101994;5102009;5102050;5102055;5102056;5102077;5102090;5102113;5102155;5102156;5102159;5102168</t>
-        </is>
-      </c>
-      <c r="L192" t="inlineStr">
-        <is>
-          <t>5101947</t>
-        </is>
-      </c>
-      <c r="M192" t="inlineStr">
-        <is>
-          <t>lines 3 and 6 resolve uniquely to serials 5101945 and 5101948; of this line's 80 candidates exactly one, 5101947, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr"/>
+      <c r="M192" t="inlineStr"/>
       <c r="N192" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 80 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O192" t="inlineStr">
@@ -11933,14 +11909,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H194" t="inlineStr">
-        <is>
-          <t>5101949</t>
-        </is>
-      </c>
+      <c r="H194" t="inlineStr"/>
       <c r="I194" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J194" t="n">
@@ -11951,7 +11923,7 @@
       <c r="M194" t="inlineStr"/>
       <c r="N194" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O194" t="inlineStr">
@@ -12003,19 +11975,11 @@
       </c>
       <c r="K195" t="inlineStr">
         <is>
-          <t>5101920;5101950</t>
-        </is>
-      </c>
-      <c r="L195" t="inlineStr">
-        <is>
-          <t>5101950</t>
-        </is>
-      </c>
-      <c r="M195" t="inlineStr">
-        <is>
-          <t>lines 7 and 9 resolve uniquely to serials 5101949 and 5101951; of this line's 2 candidates exactly one, 5101950, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+          <t>5101920;5102095</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr"/>
+      <c r="M195" t="inlineStr"/>
       <c r="N195" t="inlineStr">
         <is>
           <t>the fingerprint over 24 columns matches 2 IPUMS households and does not distinguish them; no serial is attached</t>
@@ -12059,14 +12023,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H196" t="inlineStr">
-        <is>
-          <t>5101951</t>
-        </is>
-      </c>
+      <c r="H196" t="inlineStr"/>
       <c r="I196" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J196" t="n">
@@ -12077,7 +12037,7 @@
       <c r="M196" t="inlineStr"/>
       <c r="N196" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O196" t="inlineStr">
@@ -12239,7 +12199,7 @@
       <c r="H199" t="inlineStr"/>
       <c r="I199" t="inlineStr">
         <is>
-          <t>ambiguous(80)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J199" t="n">
@@ -12247,7 +12207,7 @@
       </c>
       <c r="K199" t="inlineStr">
         <is>
-          <t>5101273;5101279;5101291;5101294;5101321;5101324;5101337;5101385;5101432;5101434;5101443;5101464;5101465;5101476;5101479;5101485;5101540;5101551;5101552;5101589;5101606;5101609;5101631;5101656;5101663;5101669;5101678;5101684;5101685;5101689;5101708;5101710;5101723;5101726;5101739;5101743;5101744;5101759;5101764;5101765;5101779;5101780;5101784;5101792;5101794;5101807;5101808;5101812;5101820;5101822;5101842;5101853;5101873;5101880;5101882;5101883;5101898;5101906;5101918;5101928;5101935;5101947;5101954;5101956;5101980;5101985;5101986;5101990;5101994;5102009;5102050;5102055;5102056;5102077;5102090;5102113;5102155;5102156;5102159;5102168</t>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
         </is>
       </c>
       <c r="L199" t="inlineStr">
@@ -12257,12 +12217,12 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>lines 11 and 13 resolve uniquely to serials 5101953 and 5101955; of this line's 80 candidates exactly one, 5101954, lies in that run at exactly the position an unbroken run would put it</t>
+          <t>lines 11 and 13 resolve uniquely to serials 5101953 and 5101955; of this line's 76 candidates exactly one, 5101954, lies in that run at exactly the position an unbroken run would put it</t>
         </is>
       </c>
       <c r="N199" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 80 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O199" t="inlineStr">
@@ -12365,7 +12325,7 @@
       <c r="H201" t="inlineStr"/>
       <c r="I201" t="inlineStr">
         <is>
-          <t>ambiguous(80)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J201" t="n">
@@ -12373,7 +12333,7 @@
       </c>
       <c r="K201" t="inlineStr">
         <is>
-          <t>5101273;5101279;5101291;5101294;5101321;5101324;5101337;5101385;5101432;5101434;5101443;5101464;5101465;5101476;5101479;5101485;5101540;5101551;5101552;5101589;5101606;5101609;5101631;5101656;5101663;5101669;5101678;5101684;5101685;5101689;5101708;5101710;5101723;5101726;5101739;5101743;5101744;5101759;5101764;5101765;5101779;5101780;5101784;5101792;5101794;5101807;5101808;5101812;5101820;5101822;5101842;5101853;5101873;5101880;5101882;5101883;5101898;5101906;5101918;5101928;5101935;5101947;5101954;5101956;5101980;5101985;5101986;5101990;5101994;5102009;5102050;5102055;5102056;5102077;5102090;5102113;5102155;5102156;5102159;5102168</t>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
         </is>
       </c>
       <c r="L201" t="inlineStr">
@@ -12383,12 +12343,12 @@
       </c>
       <c r="M201" t="inlineStr">
         <is>
-          <t>lines 13 and 16 resolve uniquely to serials 5101955 and 5101958; of this line's 80 candidates exactly one, 5101956, lies in that run at exactly the position an unbroken run would put it</t>
+          <t>lines 13 and 16 resolve uniquely to serials 5101955 and 5101958; of this line's 76 candidates exactly one, 5101956, lies in that run at exactly the position an unbroken run would put it</t>
         </is>
       </c>
       <c r="N201" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 80 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O201" t="inlineStr">
@@ -12432,7 +12392,7 @@
       <c r="H202" t="inlineStr"/>
       <c r="I202" t="inlineStr">
         <is>
-          <t>ambiguous(2)</t>
+          <t>ambiguous(3)</t>
         </is>
       </c>
       <c r="J202" t="n">
@@ -12440,22 +12400,14 @@
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>5101616;5101957</t>
-        </is>
-      </c>
-      <c r="L202" t="inlineStr">
-        <is>
-          <t>5101957</t>
-        </is>
-      </c>
-      <c r="M202" t="inlineStr">
-        <is>
-          <t>lines 13 and 16 resolve uniquely to serials 5101955 and 5101958; of this line's 2 candidates exactly one, 5101957, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+          <t>5101341;5101581;5101616</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr"/>
+      <c r="M202" t="inlineStr"/>
       <c r="N202" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 2 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 3 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O202" t="inlineStr">
@@ -12614,14 +12566,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H205" t="inlineStr">
-        <is>
-          <t>5101930</t>
-        </is>
-      </c>
+      <c r="H205" t="inlineStr"/>
       <c r="I205" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J205" t="n">
@@ -12632,7 +12580,7 @@
       <c r="M205" t="inlineStr"/>
       <c r="N205" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O205" t="inlineStr">
@@ -12673,25 +12621,33 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H206" t="inlineStr">
-        <is>
-          <t>5101931</t>
-        </is>
-      </c>
+      <c r="H206" t="inlineStr"/>
       <c r="I206" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>ambiguous(2)</t>
         </is>
       </c>
       <c r="J206" t="n">
         <v>24</v>
       </c>
-      <c r="K206" t="inlineStr"/>
-      <c r="L206" t="inlineStr"/>
-      <c r="M206" t="inlineStr"/>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>5101649;5101931</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>5101931</t>
+        </is>
+      </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>lines 17 and 21 resolve uniquely to serials 5101929 and 5101933; of this line's 2 candidates exactly one, 5101931, lies in that run at exactly the position an unbroken run would put it</t>
+        </is>
+      </c>
       <c r="N206" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>the fingerprint over 24 columns matches 2 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O206" t="inlineStr">
@@ -12732,14 +12688,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H207" t="inlineStr">
-        <is>
-          <t>5101932</t>
-        </is>
-      </c>
+      <c r="H207" t="inlineStr"/>
       <c r="I207" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J207" t="n">
@@ -12750,7 +12702,7 @@
       <c r="M207" t="inlineStr"/>
       <c r="N207" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O207" t="inlineStr">
@@ -12853,30 +12805,18 @@
       <c r="H209" t="inlineStr"/>
       <c r="I209" t="inlineStr">
         <is>
-          <t>ambiguous(2)</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J209" t="n">
         <v>24</v>
       </c>
-      <c r="K209" t="inlineStr">
-        <is>
-          <t>5101709;5101934</t>
-        </is>
-      </c>
-      <c r="L209" t="inlineStr">
-        <is>
-          <t>5101934</t>
-        </is>
-      </c>
-      <c r="M209" t="inlineStr">
-        <is>
-          <t>lines 21 and 24 resolve uniquely to serials 5101933 and 5101936; of this line's 2 candidates exactly one, 5101934, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+      <c r="K209" t="inlineStr"/>
+      <c r="L209" t="inlineStr"/>
+      <c r="M209" t="inlineStr"/>
       <c r="N209" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 2 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>contested: serial 5101709 is the sole fingerprint match for 2 different lines (33S7-9YYJ-2T line 15, 33S7-9YYJ-9M5 line 22), and a serial may not be attached twice, so none of them keeps it</t>
         </is>
       </c>
       <c r="O209" t="inlineStr">
@@ -12920,7 +12860,7 @@
       <c r="H210" t="inlineStr"/>
       <c r="I210" t="inlineStr">
         <is>
-          <t>ambiguous(80)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J210" t="n">
@@ -12928,22 +12868,18 @@
       </c>
       <c r="K210" t="inlineStr">
         <is>
-          <t>5101273;5101279;5101291;5101294;5101321;5101324;5101337;5101385;5101432;5101434;5101443;5101464;5101465;5101476;5101479;5101485;5101540;5101551;5101552;5101589;5101606;5101609;5101631;5101656;5101663;5101669;5101678;5101684;5101685;5101689;5101708;5101710;5101723;5101726;5101739;5101743;5101744;5101759;5101764;5101765;5101779;5101780;5101784;5101792;5101794;5101807;5101808;5101812;5101820;5101822;5101842;5101853;5101873;5101880;5101882;5101883;5101898;5101906;5101918;5101928;5101935;5101947;5101954;5101956;5101980;5101985;5101986;5101990;5101994;5102009;5102050;5102055;5102056;5102077;5102090;5102113;5102155;5102156;5102159;5102168</t>
-        </is>
-      </c>
-      <c r="L210" t="inlineStr">
-        <is>
-          <t>5101935</t>
-        </is>
-      </c>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr"/>
       <c r="M210" t="inlineStr">
         <is>
-          <t>lines 21 and 24 resolve uniquely to serials 5101933 and 5101936; of this line's 80 candidates exactly one, 5101935, lies in that run at exactly the position an unbroken run would put it</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 24 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N210" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 80 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O210" t="inlineStr">
@@ -12984,14 +12920,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H211" t="inlineStr">
-        <is>
-          <t>5101936</t>
-        </is>
-      </c>
+      <c r="H211" t="inlineStr"/>
       <c r="I211" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J211" t="n">
@@ -13002,7 +12934,7 @@
       <c r="M211" t="inlineStr"/>
       <c r="N211" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O211" t="inlineStr">
@@ -13046,7 +12978,7 @@
       <c r="H212" t="inlineStr"/>
       <c r="I212" t="inlineStr">
         <is>
-          <t>ambiguous(33)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J212" t="n">
@@ -13054,18 +12986,18 @@
       </c>
       <c r="K212" t="inlineStr">
         <is>
-          <t>5101309;5101427;5101502;5101537;5101555;5101557;5101583;5101648;5101653;5101682;5101702;5101722;5101813;5101827;5101864;5101869;5101890;5101895;5101905;5101909;5101937;5101939;5101946;5101973;5102000;5102011;5102038;5102044;5102052;5102105;5102109;5102144;5102187</t>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
         </is>
       </c>
       <c r="L212" t="inlineStr"/>
       <c r="M212" t="inlineStr">
         <is>
-          <t>lines 24 and 30 resolve uniquely to serials 5101936 and 5101943, and 2 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 24 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N212" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 33 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O212" t="inlineStr">
@@ -13164,7 +13096,7 @@
       <c r="H214" t="inlineStr"/>
       <c r="I214" t="inlineStr">
         <is>
-          <t>ambiguous(33)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J214" t="n">
@@ -13172,18 +13104,18 @@
       </c>
       <c r="K214" t="inlineStr">
         <is>
-          <t>5101309;5101427;5101502;5101537;5101555;5101557;5101583;5101648;5101653;5101682;5101702;5101722;5101813;5101827;5101864;5101869;5101890;5101895;5101905;5101909;5101937;5101939;5101946;5101973;5102000;5102011;5102038;5102044;5102052;5102105;5102109;5102144;5102187</t>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
         </is>
       </c>
       <c r="L214" t="inlineStr"/>
       <c r="M214" t="inlineStr">
         <is>
-          <t>lines 24 and 30 resolve uniquely to serials 5101936 and 5101943, and 2 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 24 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N214" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 33 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O214" t="inlineStr">
@@ -13227,7 +13159,7 @@
       <c r="H215" t="inlineStr"/>
       <c r="I215" t="inlineStr">
         <is>
-          <t>ambiguous(4)</t>
+          <t>ambiguous(9)</t>
         </is>
       </c>
       <c r="J215" t="n">
@@ -13235,22 +13167,18 @@
       </c>
       <c r="K215" t="inlineStr">
         <is>
-          <t>5101927;5101940;5102018;5102019</t>
-        </is>
-      </c>
-      <c r="L215" t="inlineStr">
-        <is>
-          <t>5101940</t>
-        </is>
-      </c>
+          <t>5101292;5101334;5101471;5101927;5101940;5102018;5102019;5102025;5102134</t>
+        </is>
+      </c>
+      <c r="L215" t="inlineStr"/>
       <c r="M215" t="inlineStr">
         <is>
-          <t>lines 24 and 30 resolve uniquely to serials 5101936 and 5101943; of this line's 4 candidates exactly one, 5101940, lies in that run at exactly the position an unbroken run would put it</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 2 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N215" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 4 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 9 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O215" t="inlineStr">
@@ -13294,7 +13222,7 @@
       <c r="H216" t="inlineStr"/>
       <c r="I216" t="inlineStr">
         <is>
-          <t>ambiguous(7)</t>
+          <t>ambiguous(4)</t>
         </is>
       </c>
       <c r="J216" t="n">
@@ -13302,22 +13230,18 @@
       </c>
       <c r="K216" t="inlineStr">
         <is>
-          <t>5101258;5101278;5101331;5101425;5101910;5101942;5101983</t>
-        </is>
-      </c>
-      <c r="L216" t="inlineStr">
-        <is>
-          <t>5101942</t>
-        </is>
-      </c>
+          <t>5101306;5101425;5101910;5101913</t>
+        </is>
+      </c>
+      <c r="L216" t="inlineStr"/>
       <c r="M216" t="inlineStr">
         <is>
-          <t>lines 24 and 30 resolve uniquely to serials 5101936 and 5101943; of this line's 7 candidates exactly one, 5101942, lies in that run, and an unbroken run would put this line at 5101941</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 2 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N216" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 7 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 4 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O216" t="inlineStr">

</xml_diff>

<commit_message>
T-0762: 33S7-9YYJ-VJ read line by line — three columns close, the TOTAL footing does not
</commit_message>
<xml_diff>
--- a/chicago/reference/census1840/validation/T-0504_1840_name_serial_crosswalk.xlsx
+++ b/chicago/reference/census1840/validation/T-0504_1840_name_serial_crosswalk.xlsx
@@ -1395,14 +1395,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>5101709</t>
-        </is>
-      </c>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J16" t="n">
@@ -1413,7 +1409,7 @@
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>contested: serial 5101709 is the sole fingerprint match for 2 different lines (33S7-9YYJ-2T line 15, 33S7-9YYJ-9M5 line 22), and a serial may not be attached twice, so none of them keeps it</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -11566,7 +11562,7 @@
       <c r="H188" t="inlineStr"/>
       <c r="I188" t="inlineStr">
         <is>
-          <t>ambiguous(14)</t>
+          <t>ambiguous(8)</t>
         </is>
       </c>
       <c r="J188" t="n">
@@ -11574,14 +11570,14 @@
       </c>
       <c r="K188" t="inlineStr">
         <is>
-          <t>5101354;5101370;5101379;5101712;5101732;5101757;5101821;5101896;5101924;5101941;5102016;5102149;5102154;5102164</t>
+          <t>5101712;5101821;5101896;5101924;5101941;5102149;5102154;5102164</t>
         </is>
       </c>
       <c r="L188" t="inlineStr"/>
       <c r="M188" t="inlineStr"/>
       <c r="N188" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 14 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 8 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O188" t="inlineStr">
@@ -11625,7 +11621,7 @@
       <c r="H189" t="inlineStr"/>
       <c r="I189" t="inlineStr">
         <is>
-          <t>ambiguous(24)</t>
+          <t>ambiguous(29)</t>
         </is>
       </c>
       <c r="J189" t="n">
@@ -11633,14 +11629,14 @@
       </c>
       <c r="K189" t="inlineStr">
         <is>
-          <t>5101307;5101362;5101440;5101450;5101509;5101516;5101580;5101628;5101650;5101654;5101655;5101728;5101776;5101783;5101852;5101857;5101944;5101969;5101976;5102005;5102045;5102094;5102137;5102157</t>
+          <t>5101254;5101263;5101344;5101362;5101450;5101478;5101509;5101516;5101561;5101580;5101628;5101650;5101654;5101655;5101691;5101735;5101776;5101783;5101800;5101805;5101857;5101871;5101878;5101881;5101969;5102045;5102108;5102148;5102160</t>
         </is>
       </c>
       <c r="L189" t="inlineStr"/>
       <c r="M189" t="inlineStr"/>
       <c r="N189" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 24 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 29 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O189" t="inlineStr">
@@ -11681,14 +11677,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H190" t="inlineStr">
-        <is>
-          <t>5101945</t>
-        </is>
-      </c>
+      <c r="H190" t="inlineStr"/>
       <c r="I190" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J190" t="n">
@@ -11699,7 +11691,7 @@
       <c r="M190" t="inlineStr"/>
       <c r="N190" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O190" t="inlineStr">
@@ -11743,7 +11735,7 @@
       <c r="H191" t="inlineStr"/>
       <c r="I191" t="inlineStr">
         <is>
-          <t>ambiguous(33)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J191" t="n">
@@ -11751,22 +11743,14 @@
       </c>
       <c r="K191" t="inlineStr">
         <is>
-          <t>5101309;5101427;5101502;5101537;5101555;5101557;5101583;5101648;5101653;5101682;5101702;5101722;5101813;5101827;5101864;5101869;5101890;5101895;5101905;5101909;5101937;5101939;5101946;5101973;5102000;5102011;5102038;5102044;5102052;5102105;5102109;5102144;5102187</t>
-        </is>
-      </c>
-      <c r="L191" t="inlineStr">
-        <is>
-          <t>5101946</t>
-        </is>
-      </c>
-      <c r="M191" t="inlineStr">
-        <is>
-          <t>lines 3 and 6 resolve uniquely to serials 5101945 and 5101948; of this line's 33 candidates exactly one, 5101946, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
+        </is>
+      </c>
+      <c r="L191" t="inlineStr"/>
+      <c r="M191" t="inlineStr"/>
       <c r="N191" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 33 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O191" t="inlineStr">
@@ -11810,7 +11794,7 @@
       <c r="H192" t="inlineStr"/>
       <c r="I192" t="inlineStr">
         <is>
-          <t>ambiguous(80)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J192" t="n">
@@ -11818,22 +11802,14 @@
       </c>
       <c r="K192" t="inlineStr">
         <is>
-          <t>5101273;5101279;5101291;5101294;5101321;5101324;5101337;5101385;5101432;5101434;5101443;5101464;5101465;5101476;5101479;5101485;5101540;5101551;5101552;5101589;5101606;5101609;5101631;5101656;5101663;5101669;5101678;5101684;5101685;5101689;5101708;5101710;5101723;5101726;5101739;5101743;5101744;5101759;5101764;5101765;5101779;5101780;5101784;5101792;5101794;5101807;5101808;5101812;5101820;5101822;5101842;5101853;5101873;5101880;5101882;5101883;5101898;5101906;5101918;5101928;5101935;5101947;5101954;5101956;5101980;5101985;5101986;5101990;5101994;5102009;5102050;5102055;5102056;5102077;5102090;5102113;5102155;5102156;5102159;5102168</t>
-        </is>
-      </c>
-      <c r="L192" t="inlineStr">
-        <is>
-          <t>5101947</t>
-        </is>
-      </c>
-      <c r="M192" t="inlineStr">
-        <is>
-          <t>lines 3 and 6 resolve uniquely to serials 5101945 and 5101948; of this line's 80 candidates exactly one, 5101947, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr"/>
+      <c r="M192" t="inlineStr"/>
       <c r="N192" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 80 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O192" t="inlineStr">
@@ -11933,14 +11909,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H194" t="inlineStr">
-        <is>
-          <t>5101949</t>
-        </is>
-      </c>
+      <c r="H194" t="inlineStr"/>
       <c r="I194" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J194" t="n">
@@ -11951,7 +11923,7 @@
       <c r="M194" t="inlineStr"/>
       <c r="N194" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O194" t="inlineStr">
@@ -12003,19 +11975,11 @@
       </c>
       <c r="K195" t="inlineStr">
         <is>
-          <t>5101920;5101950</t>
-        </is>
-      </c>
-      <c r="L195" t="inlineStr">
-        <is>
-          <t>5101950</t>
-        </is>
-      </c>
-      <c r="M195" t="inlineStr">
-        <is>
-          <t>lines 7 and 9 resolve uniquely to serials 5101949 and 5101951; of this line's 2 candidates exactly one, 5101950, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+          <t>5101920;5102095</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr"/>
+      <c r="M195" t="inlineStr"/>
       <c r="N195" t="inlineStr">
         <is>
           <t>the fingerprint over 24 columns matches 2 IPUMS households and does not distinguish them; no serial is attached</t>
@@ -12059,14 +12023,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H196" t="inlineStr">
-        <is>
-          <t>5101951</t>
-        </is>
-      </c>
+      <c r="H196" t="inlineStr"/>
       <c r="I196" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J196" t="n">
@@ -12077,7 +12037,7 @@
       <c r="M196" t="inlineStr"/>
       <c r="N196" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O196" t="inlineStr">
@@ -12239,7 +12199,7 @@
       <c r="H199" t="inlineStr"/>
       <c r="I199" t="inlineStr">
         <is>
-          <t>ambiguous(80)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J199" t="n">
@@ -12247,7 +12207,7 @@
       </c>
       <c r="K199" t="inlineStr">
         <is>
-          <t>5101273;5101279;5101291;5101294;5101321;5101324;5101337;5101385;5101432;5101434;5101443;5101464;5101465;5101476;5101479;5101485;5101540;5101551;5101552;5101589;5101606;5101609;5101631;5101656;5101663;5101669;5101678;5101684;5101685;5101689;5101708;5101710;5101723;5101726;5101739;5101743;5101744;5101759;5101764;5101765;5101779;5101780;5101784;5101792;5101794;5101807;5101808;5101812;5101820;5101822;5101842;5101853;5101873;5101880;5101882;5101883;5101898;5101906;5101918;5101928;5101935;5101947;5101954;5101956;5101980;5101985;5101986;5101990;5101994;5102009;5102050;5102055;5102056;5102077;5102090;5102113;5102155;5102156;5102159;5102168</t>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
         </is>
       </c>
       <c r="L199" t="inlineStr">
@@ -12257,12 +12217,12 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>lines 11 and 13 resolve uniquely to serials 5101953 and 5101955; of this line's 80 candidates exactly one, 5101954, lies in that run at exactly the position an unbroken run would put it</t>
+          <t>lines 11 and 13 resolve uniquely to serials 5101953 and 5101955; of this line's 76 candidates exactly one, 5101954, lies in that run at exactly the position an unbroken run would put it</t>
         </is>
       </c>
       <c r="N199" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 80 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O199" t="inlineStr">
@@ -12365,7 +12325,7 @@
       <c r="H201" t="inlineStr"/>
       <c r="I201" t="inlineStr">
         <is>
-          <t>ambiguous(80)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J201" t="n">
@@ -12373,7 +12333,7 @@
       </c>
       <c r="K201" t="inlineStr">
         <is>
-          <t>5101273;5101279;5101291;5101294;5101321;5101324;5101337;5101385;5101432;5101434;5101443;5101464;5101465;5101476;5101479;5101485;5101540;5101551;5101552;5101589;5101606;5101609;5101631;5101656;5101663;5101669;5101678;5101684;5101685;5101689;5101708;5101710;5101723;5101726;5101739;5101743;5101744;5101759;5101764;5101765;5101779;5101780;5101784;5101792;5101794;5101807;5101808;5101812;5101820;5101822;5101842;5101853;5101873;5101880;5101882;5101883;5101898;5101906;5101918;5101928;5101935;5101947;5101954;5101956;5101980;5101985;5101986;5101990;5101994;5102009;5102050;5102055;5102056;5102077;5102090;5102113;5102155;5102156;5102159;5102168</t>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
         </is>
       </c>
       <c r="L201" t="inlineStr">
@@ -12383,12 +12343,12 @@
       </c>
       <c r="M201" t="inlineStr">
         <is>
-          <t>lines 13 and 16 resolve uniquely to serials 5101955 and 5101958; of this line's 80 candidates exactly one, 5101956, lies in that run at exactly the position an unbroken run would put it</t>
+          <t>lines 13 and 16 resolve uniquely to serials 5101955 and 5101958; of this line's 76 candidates exactly one, 5101956, lies in that run at exactly the position an unbroken run would put it</t>
         </is>
       </c>
       <c r="N201" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 80 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O201" t="inlineStr">
@@ -12432,7 +12392,7 @@
       <c r="H202" t="inlineStr"/>
       <c r="I202" t="inlineStr">
         <is>
-          <t>ambiguous(2)</t>
+          <t>ambiguous(3)</t>
         </is>
       </c>
       <c r="J202" t="n">
@@ -12440,22 +12400,14 @@
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>5101616;5101957</t>
-        </is>
-      </c>
-      <c r="L202" t="inlineStr">
-        <is>
-          <t>5101957</t>
-        </is>
-      </c>
-      <c r="M202" t="inlineStr">
-        <is>
-          <t>lines 13 and 16 resolve uniquely to serials 5101955 and 5101958; of this line's 2 candidates exactly one, 5101957, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+          <t>5101341;5101581;5101616</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr"/>
+      <c r="M202" t="inlineStr"/>
       <c r="N202" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 2 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 3 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O202" t="inlineStr">
@@ -12614,14 +12566,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H205" t="inlineStr">
-        <is>
-          <t>5101930</t>
-        </is>
-      </c>
+      <c r="H205" t="inlineStr"/>
       <c r="I205" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J205" t="n">
@@ -12632,7 +12580,7 @@
       <c r="M205" t="inlineStr"/>
       <c r="N205" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O205" t="inlineStr">
@@ -12673,25 +12621,33 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H206" t="inlineStr">
-        <is>
-          <t>5101931</t>
-        </is>
-      </c>
+      <c r="H206" t="inlineStr"/>
       <c r="I206" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>ambiguous(2)</t>
         </is>
       </c>
       <c r="J206" t="n">
         <v>24</v>
       </c>
-      <c r="K206" t="inlineStr"/>
-      <c r="L206" t="inlineStr"/>
-      <c r="M206" t="inlineStr"/>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>5101649;5101931</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>5101931</t>
+        </is>
+      </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>lines 17 and 21 resolve uniquely to serials 5101929 and 5101933; of this line's 2 candidates exactly one, 5101931, lies in that run at exactly the position an unbroken run would put it</t>
+        </is>
+      </c>
       <c r="N206" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>the fingerprint over 24 columns matches 2 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O206" t="inlineStr">
@@ -12732,14 +12688,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H207" t="inlineStr">
-        <is>
-          <t>5101932</t>
-        </is>
-      </c>
+      <c r="H207" t="inlineStr"/>
       <c r="I207" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J207" t="n">
@@ -12750,7 +12702,7 @@
       <c r="M207" t="inlineStr"/>
       <c r="N207" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O207" t="inlineStr">
@@ -12853,30 +12805,18 @@
       <c r="H209" t="inlineStr"/>
       <c r="I209" t="inlineStr">
         <is>
-          <t>ambiguous(2)</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J209" t="n">
         <v>24</v>
       </c>
-      <c r="K209" t="inlineStr">
-        <is>
-          <t>5101709;5101934</t>
-        </is>
-      </c>
-      <c r="L209" t="inlineStr">
-        <is>
-          <t>5101934</t>
-        </is>
-      </c>
-      <c r="M209" t="inlineStr">
-        <is>
-          <t>lines 21 and 24 resolve uniquely to serials 5101933 and 5101936; of this line's 2 candidates exactly one, 5101934, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+      <c r="K209" t="inlineStr"/>
+      <c r="L209" t="inlineStr"/>
+      <c r="M209" t="inlineStr"/>
       <c r="N209" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 2 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>contested: serial 5101709 is the sole fingerprint match for 2 different lines (33S7-9YYJ-2T line 15, 33S7-9YYJ-9M5 line 22), and a serial may not be attached twice, so none of them keeps it</t>
         </is>
       </c>
       <c r="O209" t="inlineStr">
@@ -12920,7 +12860,7 @@
       <c r="H210" t="inlineStr"/>
       <c r="I210" t="inlineStr">
         <is>
-          <t>ambiguous(80)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J210" t="n">
@@ -12928,22 +12868,18 @@
       </c>
       <c r="K210" t="inlineStr">
         <is>
-          <t>5101273;5101279;5101291;5101294;5101321;5101324;5101337;5101385;5101432;5101434;5101443;5101464;5101465;5101476;5101479;5101485;5101540;5101551;5101552;5101589;5101606;5101609;5101631;5101656;5101663;5101669;5101678;5101684;5101685;5101689;5101708;5101710;5101723;5101726;5101739;5101743;5101744;5101759;5101764;5101765;5101779;5101780;5101784;5101792;5101794;5101807;5101808;5101812;5101820;5101822;5101842;5101853;5101873;5101880;5101882;5101883;5101898;5101906;5101918;5101928;5101935;5101947;5101954;5101956;5101980;5101985;5101986;5101990;5101994;5102009;5102050;5102055;5102056;5102077;5102090;5102113;5102155;5102156;5102159;5102168</t>
-        </is>
-      </c>
-      <c r="L210" t="inlineStr">
-        <is>
-          <t>5101935</t>
-        </is>
-      </c>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr"/>
       <c r="M210" t="inlineStr">
         <is>
-          <t>lines 21 and 24 resolve uniquely to serials 5101933 and 5101936; of this line's 80 candidates exactly one, 5101935, lies in that run at exactly the position an unbroken run would put it</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 24 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N210" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 80 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O210" t="inlineStr">
@@ -12984,14 +12920,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H211" t="inlineStr">
-        <is>
-          <t>5101936</t>
-        </is>
-      </c>
+      <c r="H211" t="inlineStr"/>
       <c r="I211" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J211" t="n">
@@ -13002,7 +12934,7 @@
       <c r="M211" t="inlineStr"/>
       <c r="N211" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O211" t="inlineStr">
@@ -13046,7 +12978,7 @@
       <c r="H212" t="inlineStr"/>
       <c r="I212" t="inlineStr">
         <is>
-          <t>ambiguous(33)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J212" t="n">
@@ -13054,18 +12986,18 @@
       </c>
       <c r="K212" t="inlineStr">
         <is>
-          <t>5101309;5101427;5101502;5101537;5101555;5101557;5101583;5101648;5101653;5101682;5101702;5101722;5101813;5101827;5101864;5101869;5101890;5101895;5101905;5101909;5101937;5101939;5101946;5101973;5102000;5102011;5102038;5102044;5102052;5102105;5102109;5102144;5102187</t>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
         </is>
       </c>
       <c r="L212" t="inlineStr"/>
       <c r="M212" t="inlineStr">
         <is>
-          <t>lines 24 and 30 resolve uniquely to serials 5101936 and 5101943, and 2 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 24 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N212" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 33 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O212" t="inlineStr">
@@ -13164,7 +13096,7 @@
       <c r="H214" t="inlineStr"/>
       <c r="I214" t="inlineStr">
         <is>
-          <t>ambiguous(33)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J214" t="n">
@@ -13172,18 +13104,18 @@
       </c>
       <c r="K214" t="inlineStr">
         <is>
-          <t>5101309;5101427;5101502;5101537;5101555;5101557;5101583;5101648;5101653;5101682;5101702;5101722;5101813;5101827;5101864;5101869;5101890;5101895;5101905;5101909;5101937;5101939;5101946;5101973;5102000;5102011;5102038;5102044;5102052;5102105;5102109;5102144;5102187</t>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
         </is>
       </c>
       <c r="L214" t="inlineStr"/>
       <c r="M214" t="inlineStr">
         <is>
-          <t>lines 24 and 30 resolve uniquely to serials 5101936 and 5101943, and 2 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 24 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N214" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 33 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O214" t="inlineStr">
@@ -13227,7 +13159,7 @@
       <c r="H215" t="inlineStr"/>
       <c r="I215" t="inlineStr">
         <is>
-          <t>ambiguous(4)</t>
+          <t>ambiguous(9)</t>
         </is>
       </c>
       <c r="J215" t="n">
@@ -13235,22 +13167,18 @@
       </c>
       <c r="K215" t="inlineStr">
         <is>
-          <t>5101927;5101940;5102018;5102019</t>
-        </is>
-      </c>
-      <c r="L215" t="inlineStr">
-        <is>
-          <t>5101940</t>
-        </is>
-      </c>
+          <t>5101292;5101334;5101471;5101927;5101940;5102018;5102019;5102025;5102134</t>
+        </is>
+      </c>
+      <c r="L215" t="inlineStr"/>
       <c r="M215" t="inlineStr">
         <is>
-          <t>lines 24 and 30 resolve uniquely to serials 5101936 and 5101943; of this line's 4 candidates exactly one, 5101940, lies in that run at exactly the position an unbroken run would put it</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 2 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N215" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 4 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 9 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O215" t="inlineStr">
@@ -13294,7 +13222,7 @@
       <c r="H216" t="inlineStr"/>
       <c r="I216" t="inlineStr">
         <is>
-          <t>ambiguous(7)</t>
+          <t>ambiguous(4)</t>
         </is>
       </c>
       <c r="J216" t="n">
@@ -13302,22 +13230,18 @@
       </c>
       <c r="K216" t="inlineStr">
         <is>
-          <t>5101258;5101278;5101331;5101425;5101910;5101942;5101983</t>
-        </is>
-      </c>
-      <c r="L216" t="inlineStr">
-        <is>
-          <t>5101942</t>
-        </is>
-      </c>
+          <t>5101306;5101425;5101910;5101913</t>
+        </is>
+      </c>
+      <c r="L216" t="inlineStr"/>
       <c r="M216" t="inlineStr">
         <is>
-          <t>lines 24 and 30 resolve uniquely to serials 5101936 and 5101943; of this line's 7 candidates exactly one, 5101942, lies in that run, and an unbroken run would put this line at 5101941</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 2 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N216" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 7 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 4 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O216" t="inlineStr">

</xml_diff>

<commit_message>
T-0746: the derived layers the two readings move — crosswalk, identity master, civic cards, the Fergus and land-sale spends
</commit_message>
<xml_diff>
--- a/chicago/reference/census1840/validation/T-0504_1840_name_serial_crosswalk.xlsx
+++ b/chicago/reference/census1840/validation/T-0504_1840_name_serial_crosswalk.xlsx
@@ -1395,14 +1395,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>5101709</t>
-        </is>
-      </c>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J16" t="n">
@@ -1413,7 +1409,7 @@
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>contested: serial 5101709 is the sole fingerprint match for 2 different lines (33S7-9YYJ-2T line 15, 33S7-9YYJ-9M5 line 22), and a serial may not be attached twice, so none of them keeps it</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -11566,7 +11562,7 @@
       <c r="H188" t="inlineStr"/>
       <c r="I188" t="inlineStr">
         <is>
-          <t>ambiguous(14)</t>
+          <t>ambiguous(8)</t>
         </is>
       </c>
       <c r="J188" t="n">
@@ -11574,14 +11570,14 @@
       </c>
       <c r="K188" t="inlineStr">
         <is>
-          <t>5101354;5101370;5101379;5101712;5101732;5101757;5101821;5101896;5101924;5101941;5102016;5102149;5102154;5102164</t>
+          <t>5101712;5101821;5101896;5101924;5101941;5102149;5102154;5102164</t>
         </is>
       </c>
       <c r="L188" t="inlineStr"/>
       <c r="M188" t="inlineStr"/>
       <c r="N188" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 14 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 8 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O188" t="inlineStr">
@@ -11625,7 +11621,7 @@
       <c r="H189" t="inlineStr"/>
       <c r="I189" t="inlineStr">
         <is>
-          <t>ambiguous(24)</t>
+          <t>ambiguous(29)</t>
         </is>
       </c>
       <c r="J189" t="n">
@@ -11633,14 +11629,14 @@
       </c>
       <c r="K189" t="inlineStr">
         <is>
-          <t>5101307;5101362;5101440;5101450;5101509;5101516;5101580;5101628;5101650;5101654;5101655;5101728;5101776;5101783;5101852;5101857;5101944;5101969;5101976;5102005;5102045;5102094;5102137;5102157</t>
+          <t>5101254;5101263;5101344;5101362;5101450;5101478;5101509;5101516;5101561;5101580;5101628;5101650;5101654;5101655;5101691;5101735;5101776;5101783;5101800;5101805;5101857;5101871;5101878;5101881;5101969;5102045;5102108;5102148;5102160</t>
         </is>
       </c>
       <c r="L189" t="inlineStr"/>
       <c r="M189" t="inlineStr"/>
       <c r="N189" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 24 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 29 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O189" t="inlineStr">
@@ -11681,14 +11677,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H190" t="inlineStr">
-        <is>
-          <t>5101945</t>
-        </is>
-      </c>
+      <c r="H190" t="inlineStr"/>
       <c r="I190" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J190" t="n">
@@ -11699,7 +11691,7 @@
       <c r="M190" t="inlineStr"/>
       <c r="N190" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O190" t="inlineStr">
@@ -11743,7 +11735,7 @@
       <c r="H191" t="inlineStr"/>
       <c r="I191" t="inlineStr">
         <is>
-          <t>ambiguous(33)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J191" t="n">
@@ -11751,22 +11743,14 @@
       </c>
       <c r="K191" t="inlineStr">
         <is>
-          <t>5101309;5101427;5101502;5101537;5101555;5101557;5101583;5101648;5101653;5101682;5101702;5101722;5101813;5101827;5101864;5101869;5101890;5101895;5101905;5101909;5101937;5101939;5101946;5101973;5102000;5102011;5102038;5102044;5102052;5102105;5102109;5102144;5102187</t>
-        </is>
-      </c>
-      <c r="L191" t="inlineStr">
-        <is>
-          <t>5101946</t>
-        </is>
-      </c>
-      <c r="M191" t="inlineStr">
-        <is>
-          <t>lines 3 and 6 resolve uniquely to serials 5101945 and 5101948; of this line's 33 candidates exactly one, 5101946, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
+        </is>
+      </c>
+      <c r="L191" t="inlineStr"/>
+      <c r="M191" t="inlineStr"/>
       <c r="N191" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 33 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O191" t="inlineStr">
@@ -11810,7 +11794,7 @@
       <c r="H192" t="inlineStr"/>
       <c r="I192" t="inlineStr">
         <is>
-          <t>ambiguous(80)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J192" t="n">
@@ -11818,22 +11802,14 @@
       </c>
       <c r="K192" t="inlineStr">
         <is>
-          <t>5101273;5101279;5101291;5101294;5101321;5101324;5101337;5101385;5101432;5101434;5101443;5101464;5101465;5101476;5101479;5101485;5101540;5101551;5101552;5101589;5101606;5101609;5101631;5101656;5101663;5101669;5101678;5101684;5101685;5101689;5101708;5101710;5101723;5101726;5101739;5101743;5101744;5101759;5101764;5101765;5101779;5101780;5101784;5101792;5101794;5101807;5101808;5101812;5101820;5101822;5101842;5101853;5101873;5101880;5101882;5101883;5101898;5101906;5101918;5101928;5101935;5101947;5101954;5101956;5101980;5101985;5101986;5101990;5101994;5102009;5102050;5102055;5102056;5102077;5102090;5102113;5102155;5102156;5102159;5102168</t>
-        </is>
-      </c>
-      <c r="L192" t="inlineStr">
-        <is>
-          <t>5101947</t>
-        </is>
-      </c>
-      <c r="M192" t="inlineStr">
-        <is>
-          <t>lines 3 and 6 resolve uniquely to serials 5101945 and 5101948; of this line's 80 candidates exactly one, 5101947, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr"/>
+      <c r="M192" t="inlineStr"/>
       <c r="N192" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 80 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O192" t="inlineStr">
@@ -11933,14 +11909,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H194" t="inlineStr">
-        <is>
-          <t>5101949</t>
-        </is>
-      </c>
+      <c r="H194" t="inlineStr"/>
       <c r="I194" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J194" t="n">
@@ -11951,7 +11923,7 @@
       <c r="M194" t="inlineStr"/>
       <c r="N194" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O194" t="inlineStr">
@@ -12003,19 +11975,11 @@
       </c>
       <c r="K195" t="inlineStr">
         <is>
-          <t>5101920;5101950</t>
-        </is>
-      </c>
-      <c r="L195" t="inlineStr">
-        <is>
-          <t>5101950</t>
-        </is>
-      </c>
-      <c r="M195" t="inlineStr">
-        <is>
-          <t>lines 7 and 9 resolve uniquely to serials 5101949 and 5101951; of this line's 2 candidates exactly one, 5101950, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+          <t>5101920;5102095</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr"/>
+      <c r="M195" t="inlineStr"/>
       <c r="N195" t="inlineStr">
         <is>
           <t>the fingerprint over 24 columns matches 2 IPUMS households and does not distinguish them; no serial is attached</t>
@@ -12059,14 +12023,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H196" t="inlineStr">
-        <is>
-          <t>5101951</t>
-        </is>
-      </c>
+      <c r="H196" t="inlineStr"/>
       <c r="I196" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J196" t="n">
@@ -12077,7 +12037,7 @@
       <c r="M196" t="inlineStr"/>
       <c r="N196" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O196" t="inlineStr">
@@ -12239,7 +12199,7 @@
       <c r="H199" t="inlineStr"/>
       <c r="I199" t="inlineStr">
         <is>
-          <t>ambiguous(80)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J199" t="n">
@@ -12247,7 +12207,7 @@
       </c>
       <c r="K199" t="inlineStr">
         <is>
-          <t>5101273;5101279;5101291;5101294;5101321;5101324;5101337;5101385;5101432;5101434;5101443;5101464;5101465;5101476;5101479;5101485;5101540;5101551;5101552;5101589;5101606;5101609;5101631;5101656;5101663;5101669;5101678;5101684;5101685;5101689;5101708;5101710;5101723;5101726;5101739;5101743;5101744;5101759;5101764;5101765;5101779;5101780;5101784;5101792;5101794;5101807;5101808;5101812;5101820;5101822;5101842;5101853;5101873;5101880;5101882;5101883;5101898;5101906;5101918;5101928;5101935;5101947;5101954;5101956;5101980;5101985;5101986;5101990;5101994;5102009;5102050;5102055;5102056;5102077;5102090;5102113;5102155;5102156;5102159;5102168</t>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
         </is>
       </c>
       <c r="L199" t="inlineStr">
@@ -12257,12 +12217,12 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>lines 11 and 13 resolve uniquely to serials 5101953 and 5101955; of this line's 80 candidates exactly one, 5101954, lies in that run at exactly the position an unbroken run would put it</t>
+          <t>lines 11 and 13 resolve uniquely to serials 5101953 and 5101955; of this line's 76 candidates exactly one, 5101954, lies in that run at exactly the position an unbroken run would put it</t>
         </is>
       </c>
       <c r="N199" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 80 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O199" t="inlineStr">
@@ -12365,7 +12325,7 @@
       <c r="H201" t="inlineStr"/>
       <c r="I201" t="inlineStr">
         <is>
-          <t>ambiguous(80)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J201" t="n">
@@ -12373,7 +12333,7 @@
       </c>
       <c r="K201" t="inlineStr">
         <is>
-          <t>5101273;5101279;5101291;5101294;5101321;5101324;5101337;5101385;5101432;5101434;5101443;5101464;5101465;5101476;5101479;5101485;5101540;5101551;5101552;5101589;5101606;5101609;5101631;5101656;5101663;5101669;5101678;5101684;5101685;5101689;5101708;5101710;5101723;5101726;5101739;5101743;5101744;5101759;5101764;5101765;5101779;5101780;5101784;5101792;5101794;5101807;5101808;5101812;5101820;5101822;5101842;5101853;5101873;5101880;5101882;5101883;5101898;5101906;5101918;5101928;5101935;5101947;5101954;5101956;5101980;5101985;5101986;5101990;5101994;5102009;5102050;5102055;5102056;5102077;5102090;5102113;5102155;5102156;5102159;5102168</t>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
         </is>
       </c>
       <c r="L201" t="inlineStr">
@@ -12383,12 +12343,12 @@
       </c>
       <c r="M201" t="inlineStr">
         <is>
-          <t>lines 13 and 16 resolve uniquely to serials 5101955 and 5101958; of this line's 80 candidates exactly one, 5101956, lies in that run at exactly the position an unbroken run would put it</t>
+          <t>lines 13 and 16 resolve uniquely to serials 5101955 and 5101958; of this line's 76 candidates exactly one, 5101956, lies in that run at exactly the position an unbroken run would put it</t>
         </is>
       </c>
       <c r="N201" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 80 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O201" t="inlineStr">
@@ -12432,7 +12392,7 @@
       <c r="H202" t="inlineStr"/>
       <c r="I202" t="inlineStr">
         <is>
-          <t>ambiguous(2)</t>
+          <t>ambiguous(3)</t>
         </is>
       </c>
       <c r="J202" t="n">
@@ -12440,22 +12400,14 @@
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>5101616;5101957</t>
-        </is>
-      </c>
-      <c r="L202" t="inlineStr">
-        <is>
-          <t>5101957</t>
-        </is>
-      </c>
-      <c r="M202" t="inlineStr">
-        <is>
-          <t>lines 13 and 16 resolve uniquely to serials 5101955 and 5101958; of this line's 2 candidates exactly one, 5101957, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+          <t>5101341;5101581;5101616</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr"/>
+      <c r="M202" t="inlineStr"/>
       <c r="N202" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 2 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 3 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O202" t="inlineStr">
@@ -12614,14 +12566,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H205" t="inlineStr">
-        <is>
-          <t>5101930</t>
-        </is>
-      </c>
+      <c r="H205" t="inlineStr"/>
       <c r="I205" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J205" t="n">
@@ -12632,7 +12580,7 @@
       <c r="M205" t="inlineStr"/>
       <c r="N205" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O205" t="inlineStr">
@@ -12673,25 +12621,33 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H206" t="inlineStr">
-        <is>
-          <t>5101931</t>
-        </is>
-      </c>
+      <c r="H206" t="inlineStr"/>
       <c r="I206" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>ambiguous(2)</t>
         </is>
       </c>
       <c r="J206" t="n">
         <v>24</v>
       </c>
-      <c r="K206" t="inlineStr"/>
-      <c r="L206" t="inlineStr"/>
-      <c r="M206" t="inlineStr"/>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>5101649;5101931</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>5101931</t>
+        </is>
+      </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>lines 17 and 21 resolve uniquely to serials 5101929 and 5101933; of this line's 2 candidates exactly one, 5101931, lies in that run at exactly the position an unbroken run would put it</t>
+        </is>
+      </c>
       <c r="N206" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>the fingerprint over 24 columns matches 2 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O206" t="inlineStr">
@@ -12732,14 +12688,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H207" t="inlineStr">
-        <is>
-          <t>5101932</t>
-        </is>
-      </c>
+      <c r="H207" t="inlineStr"/>
       <c r="I207" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J207" t="n">
@@ -12750,7 +12702,7 @@
       <c r="M207" t="inlineStr"/>
       <c r="N207" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O207" t="inlineStr">
@@ -12853,30 +12805,18 @@
       <c r="H209" t="inlineStr"/>
       <c r="I209" t="inlineStr">
         <is>
-          <t>ambiguous(2)</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J209" t="n">
         <v>24</v>
       </c>
-      <c r="K209" t="inlineStr">
-        <is>
-          <t>5101709;5101934</t>
-        </is>
-      </c>
-      <c r="L209" t="inlineStr">
-        <is>
-          <t>5101934</t>
-        </is>
-      </c>
-      <c r="M209" t="inlineStr">
-        <is>
-          <t>lines 21 and 24 resolve uniquely to serials 5101933 and 5101936; of this line's 2 candidates exactly one, 5101934, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+      <c r="K209" t="inlineStr"/>
+      <c r="L209" t="inlineStr"/>
+      <c r="M209" t="inlineStr"/>
       <c r="N209" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 2 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>contested: serial 5101709 is the sole fingerprint match for 2 different lines (33S7-9YYJ-2T line 15, 33S7-9YYJ-9M5 line 22), and a serial may not be attached twice, so none of them keeps it</t>
         </is>
       </c>
       <c r="O209" t="inlineStr">
@@ -12920,7 +12860,7 @@
       <c r="H210" t="inlineStr"/>
       <c r="I210" t="inlineStr">
         <is>
-          <t>ambiguous(80)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J210" t="n">
@@ -12928,22 +12868,18 @@
       </c>
       <c r="K210" t="inlineStr">
         <is>
-          <t>5101273;5101279;5101291;5101294;5101321;5101324;5101337;5101385;5101432;5101434;5101443;5101464;5101465;5101476;5101479;5101485;5101540;5101551;5101552;5101589;5101606;5101609;5101631;5101656;5101663;5101669;5101678;5101684;5101685;5101689;5101708;5101710;5101723;5101726;5101739;5101743;5101744;5101759;5101764;5101765;5101779;5101780;5101784;5101792;5101794;5101807;5101808;5101812;5101820;5101822;5101842;5101853;5101873;5101880;5101882;5101883;5101898;5101906;5101918;5101928;5101935;5101947;5101954;5101956;5101980;5101985;5101986;5101990;5101994;5102009;5102050;5102055;5102056;5102077;5102090;5102113;5102155;5102156;5102159;5102168</t>
-        </is>
-      </c>
-      <c r="L210" t="inlineStr">
-        <is>
-          <t>5101935</t>
-        </is>
-      </c>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr"/>
       <c r="M210" t="inlineStr">
         <is>
-          <t>lines 21 and 24 resolve uniquely to serials 5101933 and 5101936; of this line's 80 candidates exactly one, 5101935, lies in that run at exactly the position an unbroken run would put it</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 24 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N210" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 80 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O210" t="inlineStr">
@@ -12984,14 +12920,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H211" t="inlineStr">
-        <is>
-          <t>5101936</t>
-        </is>
-      </c>
+      <c r="H211" t="inlineStr"/>
       <c r="I211" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J211" t="n">
@@ -13002,7 +12934,7 @@
       <c r="M211" t="inlineStr"/>
       <c r="N211" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O211" t="inlineStr">
@@ -13046,7 +12978,7 @@
       <c r="H212" t="inlineStr"/>
       <c r="I212" t="inlineStr">
         <is>
-          <t>ambiguous(33)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J212" t="n">
@@ -13054,18 +12986,18 @@
       </c>
       <c r="K212" t="inlineStr">
         <is>
-          <t>5101309;5101427;5101502;5101537;5101555;5101557;5101583;5101648;5101653;5101682;5101702;5101722;5101813;5101827;5101864;5101869;5101890;5101895;5101905;5101909;5101937;5101939;5101946;5101973;5102000;5102011;5102038;5102044;5102052;5102105;5102109;5102144;5102187</t>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
         </is>
       </c>
       <c r="L212" t="inlineStr"/>
       <c r="M212" t="inlineStr">
         <is>
-          <t>lines 24 and 30 resolve uniquely to serials 5101936 and 5101943, and 2 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 24 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N212" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 33 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O212" t="inlineStr">
@@ -13164,7 +13096,7 @@
       <c r="H214" t="inlineStr"/>
       <c r="I214" t="inlineStr">
         <is>
-          <t>ambiguous(33)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J214" t="n">
@@ -13172,18 +13104,18 @@
       </c>
       <c r="K214" t="inlineStr">
         <is>
-          <t>5101309;5101427;5101502;5101537;5101555;5101557;5101583;5101648;5101653;5101682;5101702;5101722;5101813;5101827;5101864;5101869;5101890;5101895;5101905;5101909;5101937;5101939;5101946;5101973;5102000;5102011;5102038;5102044;5102052;5102105;5102109;5102144;5102187</t>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
         </is>
       </c>
       <c r="L214" t="inlineStr"/>
       <c r="M214" t="inlineStr">
         <is>
-          <t>lines 24 and 30 resolve uniquely to serials 5101936 and 5101943, and 2 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 24 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N214" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 33 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O214" t="inlineStr">
@@ -13227,7 +13159,7 @@
       <c r="H215" t="inlineStr"/>
       <c r="I215" t="inlineStr">
         <is>
-          <t>ambiguous(4)</t>
+          <t>ambiguous(9)</t>
         </is>
       </c>
       <c r="J215" t="n">
@@ -13235,22 +13167,18 @@
       </c>
       <c r="K215" t="inlineStr">
         <is>
-          <t>5101927;5101940;5102018;5102019</t>
-        </is>
-      </c>
-      <c r="L215" t="inlineStr">
-        <is>
-          <t>5101940</t>
-        </is>
-      </c>
+          <t>5101292;5101334;5101471;5101927;5101940;5102018;5102019;5102025;5102134</t>
+        </is>
+      </c>
+      <c r="L215" t="inlineStr"/>
       <c r="M215" t="inlineStr">
         <is>
-          <t>lines 24 and 30 resolve uniquely to serials 5101936 and 5101943; of this line's 4 candidates exactly one, 5101940, lies in that run at exactly the position an unbroken run would put it</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 2 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N215" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 4 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 9 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O215" t="inlineStr">
@@ -13294,7 +13222,7 @@
       <c r="H216" t="inlineStr"/>
       <c r="I216" t="inlineStr">
         <is>
-          <t>ambiguous(7)</t>
+          <t>ambiguous(4)</t>
         </is>
       </c>
       <c r="J216" t="n">
@@ -13302,22 +13230,18 @@
       </c>
       <c r="K216" t="inlineStr">
         <is>
-          <t>5101258;5101278;5101331;5101425;5101910;5101942;5101983</t>
-        </is>
-      </c>
-      <c r="L216" t="inlineStr">
-        <is>
-          <t>5101942</t>
-        </is>
-      </c>
+          <t>5101306;5101425;5101910;5101913</t>
+        </is>
+      </c>
+      <c r="L216" t="inlineStr"/>
       <c r="M216" t="inlineStr">
         <is>
-          <t>lines 24 and 30 resolve uniquely to serials 5101936 and 5101943; of this line's 7 candidates exactly one, 5101942, lies in that run, and an unbroken run would put this line at 5101941</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 2 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N216" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 7 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 4 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O216" t="inlineStr">

</xml_diff>

<commit_message>
T-0762: 33S7-9YYJ-VJ read line by line — three columns close, the footing does not (#1008)
* T-0762: claim

* T-0762: 33S7-9YYJ-VJ read line by line — the page file

* T-0762: 33S7-9YYJ-VJ read line by line — three columns close, the TOTAL footing does not

* T-0762: close the ticket on PR #1008

* T-0762: file the three smoke legs run against this diff

---------

Co-authored-by: polecat-steward <steward@polecat.live>
</commit_message>
<xml_diff>
--- a/chicago/reference/census1840/validation/T-0504_1840_name_serial_crosswalk.xlsx
+++ b/chicago/reference/census1840/validation/T-0504_1840_name_serial_crosswalk.xlsx
@@ -1395,14 +1395,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>5101709</t>
-        </is>
-      </c>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J16" t="n">
@@ -1413,7 +1409,7 @@
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>contested: serial 5101709 is the sole fingerprint match for 2 different lines (33S7-9YYJ-2T line 15, 33S7-9YYJ-9M5 line 22), and a serial may not be attached twice, so none of them keeps it</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -11566,7 +11562,7 @@
       <c r="H188" t="inlineStr"/>
       <c r="I188" t="inlineStr">
         <is>
-          <t>ambiguous(14)</t>
+          <t>ambiguous(8)</t>
         </is>
       </c>
       <c r="J188" t="n">
@@ -11574,14 +11570,14 @@
       </c>
       <c r="K188" t="inlineStr">
         <is>
-          <t>5101354;5101370;5101379;5101712;5101732;5101757;5101821;5101896;5101924;5101941;5102016;5102149;5102154;5102164</t>
+          <t>5101712;5101821;5101896;5101924;5101941;5102149;5102154;5102164</t>
         </is>
       </c>
       <c r="L188" t="inlineStr"/>
       <c r="M188" t="inlineStr"/>
       <c r="N188" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 14 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 8 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O188" t="inlineStr">
@@ -11625,7 +11621,7 @@
       <c r="H189" t="inlineStr"/>
       <c r="I189" t="inlineStr">
         <is>
-          <t>ambiguous(24)</t>
+          <t>ambiguous(29)</t>
         </is>
       </c>
       <c r="J189" t="n">
@@ -11633,14 +11629,14 @@
       </c>
       <c r="K189" t="inlineStr">
         <is>
-          <t>5101307;5101362;5101440;5101450;5101509;5101516;5101580;5101628;5101650;5101654;5101655;5101728;5101776;5101783;5101852;5101857;5101944;5101969;5101976;5102005;5102045;5102094;5102137;5102157</t>
+          <t>5101254;5101263;5101344;5101362;5101450;5101478;5101509;5101516;5101561;5101580;5101628;5101650;5101654;5101655;5101691;5101735;5101776;5101783;5101800;5101805;5101857;5101871;5101878;5101881;5101969;5102045;5102108;5102148;5102160</t>
         </is>
       </c>
       <c r="L189" t="inlineStr"/>
       <c r="M189" t="inlineStr"/>
       <c r="N189" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 24 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 29 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O189" t="inlineStr">
@@ -11681,14 +11677,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H190" t="inlineStr">
-        <is>
-          <t>5101945</t>
-        </is>
-      </c>
+      <c r="H190" t="inlineStr"/>
       <c r="I190" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J190" t="n">
@@ -11699,7 +11691,7 @@
       <c r="M190" t="inlineStr"/>
       <c r="N190" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O190" t="inlineStr">
@@ -11743,7 +11735,7 @@
       <c r="H191" t="inlineStr"/>
       <c r="I191" t="inlineStr">
         <is>
-          <t>ambiguous(33)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J191" t="n">
@@ -11751,22 +11743,14 @@
       </c>
       <c r="K191" t="inlineStr">
         <is>
-          <t>5101309;5101427;5101502;5101537;5101555;5101557;5101583;5101648;5101653;5101682;5101702;5101722;5101813;5101827;5101864;5101869;5101890;5101895;5101905;5101909;5101937;5101939;5101946;5101973;5102000;5102011;5102038;5102044;5102052;5102105;5102109;5102144;5102187</t>
-        </is>
-      </c>
-      <c r="L191" t="inlineStr">
-        <is>
-          <t>5101946</t>
-        </is>
-      </c>
-      <c r="M191" t="inlineStr">
-        <is>
-          <t>lines 3 and 6 resolve uniquely to serials 5101945 and 5101948; of this line's 33 candidates exactly one, 5101946, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
+        </is>
+      </c>
+      <c r="L191" t="inlineStr"/>
+      <c r="M191" t="inlineStr"/>
       <c r="N191" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 33 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O191" t="inlineStr">
@@ -11810,7 +11794,7 @@
       <c r="H192" t="inlineStr"/>
       <c r="I192" t="inlineStr">
         <is>
-          <t>ambiguous(80)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J192" t="n">
@@ -11818,22 +11802,14 @@
       </c>
       <c r="K192" t="inlineStr">
         <is>
-          <t>5101273;5101279;5101291;5101294;5101321;5101324;5101337;5101385;5101432;5101434;5101443;5101464;5101465;5101476;5101479;5101485;5101540;5101551;5101552;5101589;5101606;5101609;5101631;5101656;5101663;5101669;5101678;5101684;5101685;5101689;5101708;5101710;5101723;5101726;5101739;5101743;5101744;5101759;5101764;5101765;5101779;5101780;5101784;5101792;5101794;5101807;5101808;5101812;5101820;5101822;5101842;5101853;5101873;5101880;5101882;5101883;5101898;5101906;5101918;5101928;5101935;5101947;5101954;5101956;5101980;5101985;5101986;5101990;5101994;5102009;5102050;5102055;5102056;5102077;5102090;5102113;5102155;5102156;5102159;5102168</t>
-        </is>
-      </c>
-      <c r="L192" t="inlineStr">
-        <is>
-          <t>5101947</t>
-        </is>
-      </c>
-      <c r="M192" t="inlineStr">
-        <is>
-          <t>lines 3 and 6 resolve uniquely to serials 5101945 and 5101948; of this line's 80 candidates exactly one, 5101947, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr"/>
+      <c r="M192" t="inlineStr"/>
       <c r="N192" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 80 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O192" t="inlineStr">
@@ -11933,14 +11909,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H194" t="inlineStr">
-        <is>
-          <t>5101949</t>
-        </is>
-      </c>
+      <c r="H194" t="inlineStr"/>
       <c r="I194" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J194" t="n">
@@ -11951,7 +11923,7 @@
       <c r="M194" t="inlineStr"/>
       <c r="N194" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O194" t="inlineStr">
@@ -12003,19 +11975,11 @@
       </c>
       <c r="K195" t="inlineStr">
         <is>
-          <t>5101920;5101950</t>
-        </is>
-      </c>
-      <c r="L195" t="inlineStr">
-        <is>
-          <t>5101950</t>
-        </is>
-      </c>
-      <c r="M195" t="inlineStr">
-        <is>
-          <t>lines 7 and 9 resolve uniquely to serials 5101949 and 5101951; of this line's 2 candidates exactly one, 5101950, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+          <t>5101920;5102095</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr"/>
+      <c r="M195" t="inlineStr"/>
       <c r="N195" t="inlineStr">
         <is>
           <t>the fingerprint over 24 columns matches 2 IPUMS households and does not distinguish them; no serial is attached</t>
@@ -12059,14 +12023,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H196" t="inlineStr">
-        <is>
-          <t>5101951</t>
-        </is>
-      </c>
+      <c r="H196" t="inlineStr"/>
       <c r="I196" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J196" t="n">
@@ -12077,7 +12037,7 @@
       <c r="M196" t="inlineStr"/>
       <c r="N196" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O196" t="inlineStr">
@@ -12239,7 +12199,7 @@
       <c r="H199" t="inlineStr"/>
       <c r="I199" t="inlineStr">
         <is>
-          <t>ambiguous(80)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J199" t="n">
@@ -12247,7 +12207,7 @@
       </c>
       <c r="K199" t="inlineStr">
         <is>
-          <t>5101273;5101279;5101291;5101294;5101321;5101324;5101337;5101385;5101432;5101434;5101443;5101464;5101465;5101476;5101479;5101485;5101540;5101551;5101552;5101589;5101606;5101609;5101631;5101656;5101663;5101669;5101678;5101684;5101685;5101689;5101708;5101710;5101723;5101726;5101739;5101743;5101744;5101759;5101764;5101765;5101779;5101780;5101784;5101792;5101794;5101807;5101808;5101812;5101820;5101822;5101842;5101853;5101873;5101880;5101882;5101883;5101898;5101906;5101918;5101928;5101935;5101947;5101954;5101956;5101980;5101985;5101986;5101990;5101994;5102009;5102050;5102055;5102056;5102077;5102090;5102113;5102155;5102156;5102159;5102168</t>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
         </is>
       </c>
       <c r="L199" t="inlineStr">
@@ -12257,12 +12217,12 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>lines 11 and 13 resolve uniquely to serials 5101953 and 5101955; of this line's 80 candidates exactly one, 5101954, lies in that run at exactly the position an unbroken run would put it</t>
+          <t>lines 11 and 13 resolve uniquely to serials 5101953 and 5101955; of this line's 76 candidates exactly one, 5101954, lies in that run at exactly the position an unbroken run would put it</t>
         </is>
       </c>
       <c r="N199" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 80 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O199" t="inlineStr">
@@ -12365,7 +12325,7 @@
       <c r="H201" t="inlineStr"/>
       <c r="I201" t="inlineStr">
         <is>
-          <t>ambiguous(80)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J201" t="n">
@@ -12373,7 +12333,7 @@
       </c>
       <c r="K201" t="inlineStr">
         <is>
-          <t>5101273;5101279;5101291;5101294;5101321;5101324;5101337;5101385;5101432;5101434;5101443;5101464;5101465;5101476;5101479;5101485;5101540;5101551;5101552;5101589;5101606;5101609;5101631;5101656;5101663;5101669;5101678;5101684;5101685;5101689;5101708;5101710;5101723;5101726;5101739;5101743;5101744;5101759;5101764;5101765;5101779;5101780;5101784;5101792;5101794;5101807;5101808;5101812;5101820;5101822;5101842;5101853;5101873;5101880;5101882;5101883;5101898;5101906;5101918;5101928;5101935;5101947;5101954;5101956;5101980;5101985;5101986;5101990;5101994;5102009;5102050;5102055;5102056;5102077;5102090;5102113;5102155;5102156;5102159;5102168</t>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
         </is>
       </c>
       <c r="L201" t="inlineStr">
@@ -12383,12 +12343,12 @@
       </c>
       <c r="M201" t="inlineStr">
         <is>
-          <t>lines 13 and 16 resolve uniquely to serials 5101955 and 5101958; of this line's 80 candidates exactly one, 5101956, lies in that run at exactly the position an unbroken run would put it</t>
+          <t>lines 13 and 16 resolve uniquely to serials 5101955 and 5101958; of this line's 76 candidates exactly one, 5101956, lies in that run at exactly the position an unbroken run would put it</t>
         </is>
       </c>
       <c r="N201" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 80 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O201" t="inlineStr">
@@ -12432,7 +12392,7 @@
       <c r="H202" t="inlineStr"/>
       <c r="I202" t="inlineStr">
         <is>
-          <t>ambiguous(2)</t>
+          <t>ambiguous(3)</t>
         </is>
       </c>
       <c r="J202" t="n">
@@ -12440,22 +12400,14 @@
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>5101616;5101957</t>
-        </is>
-      </c>
-      <c r="L202" t="inlineStr">
-        <is>
-          <t>5101957</t>
-        </is>
-      </c>
-      <c r="M202" t="inlineStr">
-        <is>
-          <t>lines 13 and 16 resolve uniquely to serials 5101955 and 5101958; of this line's 2 candidates exactly one, 5101957, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+          <t>5101341;5101581;5101616</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr"/>
+      <c r="M202" t="inlineStr"/>
       <c r="N202" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 2 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 3 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O202" t="inlineStr">
@@ -12614,14 +12566,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H205" t="inlineStr">
-        <is>
-          <t>5101930</t>
-        </is>
-      </c>
+      <c r="H205" t="inlineStr"/>
       <c r="I205" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J205" t="n">
@@ -12632,7 +12580,7 @@
       <c r="M205" t="inlineStr"/>
       <c r="N205" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O205" t="inlineStr">
@@ -12673,25 +12621,33 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H206" t="inlineStr">
-        <is>
-          <t>5101931</t>
-        </is>
-      </c>
+      <c r="H206" t="inlineStr"/>
       <c r="I206" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>ambiguous(2)</t>
         </is>
       </c>
       <c r="J206" t="n">
         <v>24</v>
       </c>
-      <c r="K206" t="inlineStr"/>
-      <c r="L206" t="inlineStr"/>
-      <c r="M206" t="inlineStr"/>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>5101649;5101931</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>5101931</t>
+        </is>
+      </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>lines 17 and 21 resolve uniquely to serials 5101929 and 5101933; of this line's 2 candidates exactly one, 5101931, lies in that run at exactly the position an unbroken run would put it</t>
+        </is>
+      </c>
       <c r="N206" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>the fingerprint over 24 columns matches 2 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O206" t="inlineStr">
@@ -12732,14 +12688,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H207" t="inlineStr">
-        <is>
-          <t>5101932</t>
-        </is>
-      </c>
+      <c r="H207" t="inlineStr"/>
       <c r="I207" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J207" t="n">
@@ -12750,7 +12702,7 @@
       <c r="M207" t="inlineStr"/>
       <c r="N207" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O207" t="inlineStr">
@@ -12853,30 +12805,18 @@
       <c r="H209" t="inlineStr"/>
       <c r="I209" t="inlineStr">
         <is>
-          <t>ambiguous(2)</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J209" t="n">
         <v>24</v>
       </c>
-      <c r="K209" t="inlineStr">
-        <is>
-          <t>5101709;5101934</t>
-        </is>
-      </c>
-      <c r="L209" t="inlineStr">
-        <is>
-          <t>5101934</t>
-        </is>
-      </c>
-      <c r="M209" t="inlineStr">
-        <is>
-          <t>lines 21 and 24 resolve uniquely to serials 5101933 and 5101936; of this line's 2 candidates exactly one, 5101934, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+      <c r="K209" t="inlineStr"/>
+      <c r="L209" t="inlineStr"/>
+      <c r="M209" t="inlineStr"/>
       <c r="N209" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 2 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>contested: serial 5101709 is the sole fingerprint match for 2 different lines (33S7-9YYJ-2T line 15, 33S7-9YYJ-9M5 line 22), and a serial may not be attached twice, so none of them keeps it</t>
         </is>
       </c>
       <c r="O209" t="inlineStr">
@@ -12920,7 +12860,7 @@
       <c r="H210" t="inlineStr"/>
       <c r="I210" t="inlineStr">
         <is>
-          <t>ambiguous(80)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J210" t="n">
@@ -12928,22 +12868,18 @@
       </c>
       <c r="K210" t="inlineStr">
         <is>
-          <t>5101273;5101279;5101291;5101294;5101321;5101324;5101337;5101385;5101432;5101434;5101443;5101464;5101465;5101476;5101479;5101485;5101540;5101551;5101552;5101589;5101606;5101609;5101631;5101656;5101663;5101669;5101678;5101684;5101685;5101689;5101708;5101710;5101723;5101726;5101739;5101743;5101744;5101759;5101764;5101765;5101779;5101780;5101784;5101792;5101794;5101807;5101808;5101812;5101820;5101822;5101842;5101853;5101873;5101880;5101882;5101883;5101898;5101906;5101918;5101928;5101935;5101947;5101954;5101956;5101980;5101985;5101986;5101990;5101994;5102009;5102050;5102055;5102056;5102077;5102090;5102113;5102155;5102156;5102159;5102168</t>
-        </is>
-      </c>
-      <c r="L210" t="inlineStr">
-        <is>
-          <t>5101935</t>
-        </is>
-      </c>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr"/>
       <c r="M210" t="inlineStr">
         <is>
-          <t>lines 21 and 24 resolve uniquely to serials 5101933 and 5101936; of this line's 80 candidates exactly one, 5101935, lies in that run at exactly the position an unbroken run would put it</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 24 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N210" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 80 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O210" t="inlineStr">
@@ -12984,14 +12920,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H211" t="inlineStr">
-        <is>
-          <t>5101936</t>
-        </is>
-      </c>
+      <c r="H211" t="inlineStr"/>
       <c r="I211" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J211" t="n">
@@ -13002,7 +12934,7 @@
       <c r="M211" t="inlineStr"/>
       <c r="N211" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O211" t="inlineStr">
@@ -13046,7 +12978,7 @@
       <c r="H212" t="inlineStr"/>
       <c r="I212" t="inlineStr">
         <is>
-          <t>ambiguous(33)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J212" t="n">
@@ -13054,18 +12986,18 @@
       </c>
       <c r="K212" t="inlineStr">
         <is>
-          <t>5101309;5101427;5101502;5101537;5101555;5101557;5101583;5101648;5101653;5101682;5101702;5101722;5101813;5101827;5101864;5101869;5101890;5101895;5101905;5101909;5101937;5101939;5101946;5101973;5102000;5102011;5102038;5102044;5102052;5102105;5102109;5102144;5102187</t>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
         </is>
       </c>
       <c r="L212" t="inlineStr"/>
       <c r="M212" t="inlineStr">
         <is>
-          <t>lines 24 and 30 resolve uniquely to serials 5101936 and 5101943, and 2 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 24 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N212" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 33 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O212" t="inlineStr">
@@ -13164,7 +13096,7 @@
       <c r="H214" t="inlineStr"/>
       <c r="I214" t="inlineStr">
         <is>
-          <t>ambiguous(33)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J214" t="n">
@@ -13172,18 +13104,18 @@
       </c>
       <c r="K214" t="inlineStr">
         <is>
-          <t>5101309;5101427;5101502;5101537;5101555;5101557;5101583;5101648;5101653;5101682;5101702;5101722;5101813;5101827;5101864;5101869;5101890;5101895;5101905;5101909;5101937;5101939;5101946;5101973;5102000;5102011;5102038;5102044;5102052;5102105;5102109;5102144;5102187</t>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
         </is>
       </c>
       <c r="L214" t="inlineStr"/>
       <c r="M214" t="inlineStr">
         <is>
-          <t>lines 24 and 30 resolve uniquely to serials 5101936 and 5101943, and 2 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 24 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N214" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 33 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O214" t="inlineStr">
@@ -13227,7 +13159,7 @@
       <c r="H215" t="inlineStr"/>
       <c r="I215" t="inlineStr">
         <is>
-          <t>ambiguous(4)</t>
+          <t>ambiguous(9)</t>
         </is>
       </c>
       <c r="J215" t="n">
@@ -13235,22 +13167,18 @@
       </c>
       <c r="K215" t="inlineStr">
         <is>
-          <t>5101927;5101940;5102018;5102019</t>
-        </is>
-      </c>
-      <c r="L215" t="inlineStr">
-        <is>
-          <t>5101940</t>
-        </is>
-      </c>
+          <t>5101292;5101334;5101471;5101927;5101940;5102018;5102019;5102025;5102134</t>
+        </is>
+      </c>
+      <c r="L215" t="inlineStr"/>
       <c r="M215" t="inlineStr">
         <is>
-          <t>lines 24 and 30 resolve uniquely to serials 5101936 and 5101943; of this line's 4 candidates exactly one, 5101940, lies in that run at exactly the position an unbroken run would put it</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 2 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N215" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 4 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 9 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O215" t="inlineStr">
@@ -13294,7 +13222,7 @@
       <c r="H216" t="inlineStr"/>
       <c r="I216" t="inlineStr">
         <is>
-          <t>ambiguous(7)</t>
+          <t>ambiguous(4)</t>
         </is>
       </c>
       <c r="J216" t="n">
@@ -13302,22 +13230,18 @@
       </c>
       <c r="K216" t="inlineStr">
         <is>
-          <t>5101258;5101278;5101331;5101425;5101910;5101942;5101983</t>
-        </is>
-      </c>
-      <c r="L216" t="inlineStr">
-        <is>
-          <t>5101942</t>
-        </is>
-      </c>
+          <t>5101306;5101425;5101910;5101913</t>
+        </is>
+      </c>
+      <c r="L216" t="inlineStr"/>
       <c r="M216" t="inlineStr">
         <is>
-          <t>lines 24 and 30 resolve uniquely to serials 5101936 and 5101943; of this line's 7 candidates exactly one, 5101942, lies in that run, and an unbroken run would put this line at 5101941</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 2 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N216" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 7 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 4 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O216" t="inlineStr">

</xml_diff>

<commit_message>
T-0743: rebuild the serial crosswalk from the new reading; restore the four synthesizer-written mirror files; file T-0921
</commit_message>
<xml_diff>
--- a/chicago/reference/census1840/validation/T-0504_1840_name_serial_crosswalk.xlsx
+++ b/chicago/reference/census1840/validation/T-0504_1840_name_serial_crosswalk.xlsx
@@ -1395,14 +1395,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>5101709</t>
-        </is>
-      </c>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J16" t="n">
@@ -1413,7 +1409,7 @@
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>contested: serial 5101709 is the sole fingerprint match for 2 different lines (33S7-9YYJ-2T line 15, 33S7-9YYJ-9M5 line 22), and a serial may not be attached twice, so none of them keeps it</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -11566,7 +11562,7 @@
       <c r="H188" t="inlineStr"/>
       <c r="I188" t="inlineStr">
         <is>
-          <t>ambiguous(14)</t>
+          <t>ambiguous(8)</t>
         </is>
       </c>
       <c r="J188" t="n">
@@ -11574,14 +11570,14 @@
       </c>
       <c r="K188" t="inlineStr">
         <is>
-          <t>5101354;5101370;5101379;5101712;5101732;5101757;5101821;5101896;5101924;5101941;5102016;5102149;5102154;5102164</t>
+          <t>5101712;5101821;5101896;5101924;5101941;5102149;5102154;5102164</t>
         </is>
       </c>
       <c r="L188" t="inlineStr"/>
       <c r="M188" t="inlineStr"/>
       <c r="N188" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 14 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 8 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O188" t="inlineStr">
@@ -11625,7 +11621,7 @@
       <c r="H189" t="inlineStr"/>
       <c r="I189" t="inlineStr">
         <is>
-          <t>ambiguous(24)</t>
+          <t>ambiguous(29)</t>
         </is>
       </c>
       <c r="J189" t="n">
@@ -11633,14 +11629,14 @@
       </c>
       <c r="K189" t="inlineStr">
         <is>
-          <t>5101307;5101362;5101440;5101450;5101509;5101516;5101580;5101628;5101650;5101654;5101655;5101728;5101776;5101783;5101852;5101857;5101944;5101969;5101976;5102005;5102045;5102094;5102137;5102157</t>
+          <t>5101254;5101263;5101344;5101362;5101450;5101478;5101509;5101516;5101561;5101580;5101628;5101650;5101654;5101655;5101691;5101735;5101776;5101783;5101800;5101805;5101857;5101871;5101878;5101881;5101969;5102045;5102108;5102148;5102160</t>
         </is>
       </c>
       <c r="L189" t="inlineStr"/>
       <c r="M189" t="inlineStr"/>
       <c r="N189" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 24 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 29 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O189" t="inlineStr">
@@ -11681,14 +11677,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H190" t="inlineStr">
-        <is>
-          <t>5101945</t>
-        </is>
-      </c>
+      <c r="H190" t="inlineStr"/>
       <c r="I190" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J190" t="n">
@@ -11699,7 +11691,7 @@
       <c r="M190" t="inlineStr"/>
       <c r="N190" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O190" t="inlineStr">
@@ -11743,7 +11735,7 @@
       <c r="H191" t="inlineStr"/>
       <c r="I191" t="inlineStr">
         <is>
-          <t>ambiguous(33)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J191" t="n">
@@ -11751,22 +11743,14 @@
       </c>
       <c r="K191" t="inlineStr">
         <is>
-          <t>5101309;5101427;5101502;5101537;5101555;5101557;5101583;5101648;5101653;5101682;5101702;5101722;5101813;5101827;5101864;5101869;5101890;5101895;5101905;5101909;5101937;5101939;5101946;5101973;5102000;5102011;5102038;5102044;5102052;5102105;5102109;5102144;5102187</t>
-        </is>
-      </c>
-      <c r="L191" t="inlineStr">
-        <is>
-          <t>5101946</t>
-        </is>
-      </c>
-      <c r="M191" t="inlineStr">
-        <is>
-          <t>lines 3 and 6 resolve uniquely to serials 5101945 and 5101948; of this line's 33 candidates exactly one, 5101946, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
+        </is>
+      </c>
+      <c r="L191" t="inlineStr"/>
+      <c r="M191" t="inlineStr"/>
       <c r="N191" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 33 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O191" t="inlineStr">
@@ -11810,7 +11794,7 @@
       <c r="H192" t="inlineStr"/>
       <c r="I192" t="inlineStr">
         <is>
-          <t>ambiguous(80)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J192" t="n">
@@ -11818,22 +11802,14 @@
       </c>
       <c r="K192" t="inlineStr">
         <is>
-          <t>5101273;5101279;5101291;5101294;5101321;5101324;5101337;5101385;5101432;5101434;5101443;5101464;5101465;5101476;5101479;5101485;5101540;5101551;5101552;5101589;5101606;5101609;5101631;5101656;5101663;5101669;5101678;5101684;5101685;5101689;5101708;5101710;5101723;5101726;5101739;5101743;5101744;5101759;5101764;5101765;5101779;5101780;5101784;5101792;5101794;5101807;5101808;5101812;5101820;5101822;5101842;5101853;5101873;5101880;5101882;5101883;5101898;5101906;5101918;5101928;5101935;5101947;5101954;5101956;5101980;5101985;5101986;5101990;5101994;5102009;5102050;5102055;5102056;5102077;5102090;5102113;5102155;5102156;5102159;5102168</t>
-        </is>
-      </c>
-      <c r="L192" t="inlineStr">
-        <is>
-          <t>5101947</t>
-        </is>
-      </c>
-      <c r="M192" t="inlineStr">
-        <is>
-          <t>lines 3 and 6 resolve uniquely to serials 5101945 and 5101948; of this line's 80 candidates exactly one, 5101947, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr"/>
+      <c r="M192" t="inlineStr"/>
       <c r="N192" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 80 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O192" t="inlineStr">
@@ -11933,14 +11909,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H194" t="inlineStr">
-        <is>
-          <t>5101949</t>
-        </is>
-      </c>
+      <c r="H194" t="inlineStr"/>
       <c r="I194" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J194" t="n">
@@ -11951,7 +11923,7 @@
       <c r="M194" t="inlineStr"/>
       <c r="N194" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O194" t="inlineStr">
@@ -12003,19 +11975,11 @@
       </c>
       <c r="K195" t="inlineStr">
         <is>
-          <t>5101920;5101950</t>
-        </is>
-      </c>
-      <c r="L195" t="inlineStr">
-        <is>
-          <t>5101950</t>
-        </is>
-      </c>
-      <c r="M195" t="inlineStr">
-        <is>
-          <t>lines 7 and 9 resolve uniquely to serials 5101949 and 5101951; of this line's 2 candidates exactly one, 5101950, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+          <t>5101920;5102095</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr"/>
+      <c r="M195" t="inlineStr"/>
       <c r="N195" t="inlineStr">
         <is>
           <t>the fingerprint over 24 columns matches 2 IPUMS households and does not distinguish them; no serial is attached</t>
@@ -12059,14 +12023,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H196" t="inlineStr">
-        <is>
-          <t>5101951</t>
-        </is>
-      </c>
+      <c r="H196" t="inlineStr"/>
       <c r="I196" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J196" t="n">
@@ -12077,7 +12037,7 @@
       <c r="M196" t="inlineStr"/>
       <c r="N196" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O196" t="inlineStr">
@@ -12239,7 +12199,7 @@
       <c r="H199" t="inlineStr"/>
       <c r="I199" t="inlineStr">
         <is>
-          <t>ambiguous(80)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J199" t="n">
@@ -12247,7 +12207,7 @@
       </c>
       <c r="K199" t="inlineStr">
         <is>
-          <t>5101273;5101279;5101291;5101294;5101321;5101324;5101337;5101385;5101432;5101434;5101443;5101464;5101465;5101476;5101479;5101485;5101540;5101551;5101552;5101589;5101606;5101609;5101631;5101656;5101663;5101669;5101678;5101684;5101685;5101689;5101708;5101710;5101723;5101726;5101739;5101743;5101744;5101759;5101764;5101765;5101779;5101780;5101784;5101792;5101794;5101807;5101808;5101812;5101820;5101822;5101842;5101853;5101873;5101880;5101882;5101883;5101898;5101906;5101918;5101928;5101935;5101947;5101954;5101956;5101980;5101985;5101986;5101990;5101994;5102009;5102050;5102055;5102056;5102077;5102090;5102113;5102155;5102156;5102159;5102168</t>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
         </is>
       </c>
       <c r="L199" t="inlineStr">
@@ -12257,12 +12217,12 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>lines 11 and 13 resolve uniquely to serials 5101953 and 5101955; of this line's 80 candidates exactly one, 5101954, lies in that run at exactly the position an unbroken run would put it</t>
+          <t>lines 11 and 13 resolve uniquely to serials 5101953 and 5101955; of this line's 76 candidates exactly one, 5101954, lies in that run at exactly the position an unbroken run would put it</t>
         </is>
       </c>
       <c r="N199" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 80 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O199" t="inlineStr">
@@ -12365,7 +12325,7 @@
       <c r="H201" t="inlineStr"/>
       <c r="I201" t="inlineStr">
         <is>
-          <t>ambiguous(80)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J201" t="n">
@@ -12373,7 +12333,7 @@
       </c>
       <c r="K201" t="inlineStr">
         <is>
-          <t>5101273;5101279;5101291;5101294;5101321;5101324;5101337;5101385;5101432;5101434;5101443;5101464;5101465;5101476;5101479;5101485;5101540;5101551;5101552;5101589;5101606;5101609;5101631;5101656;5101663;5101669;5101678;5101684;5101685;5101689;5101708;5101710;5101723;5101726;5101739;5101743;5101744;5101759;5101764;5101765;5101779;5101780;5101784;5101792;5101794;5101807;5101808;5101812;5101820;5101822;5101842;5101853;5101873;5101880;5101882;5101883;5101898;5101906;5101918;5101928;5101935;5101947;5101954;5101956;5101980;5101985;5101986;5101990;5101994;5102009;5102050;5102055;5102056;5102077;5102090;5102113;5102155;5102156;5102159;5102168</t>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
         </is>
       </c>
       <c r="L201" t="inlineStr">
@@ -12383,12 +12343,12 @@
       </c>
       <c r="M201" t="inlineStr">
         <is>
-          <t>lines 13 and 16 resolve uniquely to serials 5101955 and 5101958; of this line's 80 candidates exactly one, 5101956, lies in that run at exactly the position an unbroken run would put it</t>
+          <t>lines 13 and 16 resolve uniquely to serials 5101955 and 5101958; of this line's 76 candidates exactly one, 5101956, lies in that run at exactly the position an unbroken run would put it</t>
         </is>
       </c>
       <c r="N201" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 80 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O201" t="inlineStr">
@@ -12432,7 +12392,7 @@
       <c r="H202" t="inlineStr"/>
       <c r="I202" t="inlineStr">
         <is>
-          <t>ambiguous(2)</t>
+          <t>ambiguous(3)</t>
         </is>
       </c>
       <c r="J202" t="n">
@@ -12440,22 +12400,14 @@
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>5101616;5101957</t>
-        </is>
-      </c>
-      <c r="L202" t="inlineStr">
-        <is>
-          <t>5101957</t>
-        </is>
-      </c>
-      <c r="M202" t="inlineStr">
-        <is>
-          <t>lines 13 and 16 resolve uniquely to serials 5101955 and 5101958; of this line's 2 candidates exactly one, 5101957, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+          <t>5101341;5101581;5101616</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr"/>
+      <c r="M202" t="inlineStr"/>
       <c r="N202" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 2 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 3 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O202" t="inlineStr">
@@ -12614,14 +12566,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H205" t="inlineStr">
-        <is>
-          <t>5101930</t>
-        </is>
-      </c>
+      <c r="H205" t="inlineStr"/>
       <c r="I205" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J205" t="n">
@@ -12632,7 +12580,7 @@
       <c r="M205" t="inlineStr"/>
       <c r="N205" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O205" t="inlineStr">
@@ -12673,25 +12621,33 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H206" t="inlineStr">
-        <is>
-          <t>5101931</t>
-        </is>
-      </c>
+      <c r="H206" t="inlineStr"/>
       <c r="I206" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>ambiguous(2)</t>
         </is>
       </c>
       <c r="J206" t="n">
         <v>24</v>
       </c>
-      <c r="K206" t="inlineStr"/>
-      <c r="L206" t="inlineStr"/>
-      <c r="M206" t="inlineStr"/>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>5101649;5101931</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>5101931</t>
+        </is>
+      </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>lines 17 and 21 resolve uniquely to serials 5101929 and 5101933; of this line's 2 candidates exactly one, 5101931, lies in that run at exactly the position an unbroken run would put it</t>
+        </is>
+      </c>
       <c r="N206" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>the fingerprint over 24 columns matches 2 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O206" t="inlineStr">
@@ -12732,14 +12688,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H207" t="inlineStr">
-        <is>
-          <t>5101932</t>
-        </is>
-      </c>
+      <c r="H207" t="inlineStr"/>
       <c r="I207" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J207" t="n">
@@ -12750,7 +12702,7 @@
       <c r="M207" t="inlineStr"/>
       <c r="N207" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O207" t="inlineStr">
@@ -12853,30 +12805,18 @@
       <c r="H209" t="inlineStr"/>
       <c r="I209" t="inlineStr">
         <is>
-          <t>ambiguous(2)</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J209" t="n">
         <v>24</v>
       </c>
-      <c r="K209" t="inlineStr">
-        <is>
-          <t>5101709;5101934</t>
-        </is>
-      </c>
-      <c r="L209" t="inlineStr">
-        <is>
-          <t>5101934</t>
-        </is>
-      </c>
-      <c r="M209" t="inlineStr">
-        <is>
-          <t>lines 21 and 24 resolve uniquely to serials 5101933 and 5101936; of this line's 2 candidates exactly one, 5101934, lies in that run at exactly the position an unbroken run would put it</t>
-        </is>
-      </c>
+      <c r="K209" t="inlineStr"/>
+      <c r="L209" t="inlineStr"/>
+      <c r="M209" t="inlineStr"/>
       <c r="N209" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 2 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>contested: serial 5101709 is the sole fingerprint match for 2 different lines (33S7-9YYJ-2T line 15, 33S7-9YYJ-9M5 line 22), and a serial may not be attached twice, so none of them keeps it</t>
         </is>
       </c>
       <c r="O209" t="inlineStr">
@@ -12920,7 +12860,7 @@
       <c r="H210" t="inlineStr"/>
       <c r="I210" t="inlineStr">
         <is>
-          <t>ambiguous(80)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J210" t="n">
@@ -12928,22 +12868,18 @@
       </c>
       <c r="K210" t="inlineStr">
         <is>
-          <t>5101273;5101279;5101291;5101294;5101321;5101324;5101337;5101385;5101432;5101434;5101443;5101464;5101465;5101476;5101479;5101485;5101540;5101551;5101552;5101589;5101606;5101609;5101631;5101656;5101663;5101669;5101678;5101684;5101685;5101689;5101708;5101710;5101723;5101726;5101739;5101743;5101744;5101759;5101764;5101765;5101779;5101780;5101784;5101792;5101794;5101807;5101808;5101812;5101820;5101822;5101842;5101853;5101873;5101880;5101882;5101883;5101898;5101906;5101918;5101928;5101935;5101947;5101954;5101956;5101980;5101985;5101986;5101990;5101994;5102009;5102050;5102055;5102056;5102077;5102090;5102113;5102155;5102156;5102159;5102168</t>
-        </is>
-      </c>
-      <c r="L210" t="inlineStr">
-        <is>
-          <t>5101935</t>
-        </is>
-      </c>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr"/>
       <c r="M210" t="inlineStr">
         <is>
-          <t>lines 21 and 24 resolve uniquely to serials 5101933 and 5101936; of this line's 80 candidates exactly one, 5101935, lies in that run at exactly the position an unbroken run would put it</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 24 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N210" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 80 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O210" t="inlineStr">
@@ -12984,14 +12920,10 @@
           <t>scan_verified</t>
         </is>
       </c>
-      <c r="H211" t="inlineStr">
-        <is>
-          <t>5101936</t>
-        </is>
-      </c>
+      <c r="H211" t="inlineStr"/>
       <c r="I211" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J211" t="n">
@@ -13002,7 +12934,7 @@
       <c r="M211" t="inlineStr"/>
       <c r="N211" t="inlineStr">
         <is>
-          <t>free-white age-band fingerprint over 24 of the schedule's 26 columns matches exactly one of the 964 IPUMS households; 2 columns masked because this page's reading does not close them against the enumerator's printed totals</t>
+          <t>no IPUMS household carries this pattern over the 24 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
         </is>
       </c>
       <c r="O211" t="inlineStr">
@@ -13046,7 +12978,7 @@
       <c r="H212" t="inlineStr"/>
       <c r="I212" t="inlineStr">
         <is>
-          <t>ambiguous(33)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J212" t="n">
@@ -13054,18 +12986,18 @@
       </c>
       <c r="K212" t="inlineStr">
         <is>
-          <t>5101309;5101427;5101502;5101537;5101555;5101557;5101583;5101648;5101653;5101682;5101702;5101722;5101813;5101827;5101864;5101869;5101890;5101895;5101905;5101909;5101937;5101939;5101946;5101973;5102000;5102011;5102038;5102044;5102052;5102105;5102109;5102144;5102187</t>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
         </is>
       </c>
       <c r="L212" t="inlineStr"/>
       <c r="M212" t="inlineStr">
         <is>
-          <t>lines 24 and 30 resolve uniquely to serials 5101936 and 5101943, and 2 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 24 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N212" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 33 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O212" t="inlineStr">
@@ -13164,7 +13096,7 @@
       <c r="H214" t="inlineStr"/>
       <c r="I214" t="inlineStr">
         <is>
-          <t>ambiguous(33)</t>
+          <t>ambiguous(76)</t>
         </is>
       </c>
       <c r="J214" t="n">
@@ -13172,18 +13104,18 @@
       </c>
       <c r="K214" t="inlineStr">
         <is>
-          <t>5101309;5101427;5101502;5101537;5101555;5101557;5101583;5101648;5101653;5101682;5101702;5101722;5101813;5101827;5101864;5101869;5101890;5101895;5101905;5101909;5101937;5101939;5101946;5101973;5102000;5102011;5102038;5102044;5102052;5102105;5102109;5102144;5102187</t>
+          <t>5101273;5101283;5101291;5101294;5101321;5101324;5101337;5101392;5101427;5101432;5101434;5101443;5101445;5101464;5101476;5101479;5101485;5101551;5101552;5101555;5101557;5101559;5101589;5101606;5101609;5101631;5101648;5101653;5101656;5101663;5101678;5101682;5101696;5101722;5101739;5101743;5101759;5101765;5101794;5101812;5101813;5101820;5101822;5101827;5101853;5101863;5101864;5101869;5101880;5101882;5101883;5101890;5101905;5101906;5101918;5101928;5101939;5101946;5101947;5101954;5101956;5101973;5101985;5101990;5102000;5102011;5102050;5102052;5102105;5102113;5102144;5102155;5102156;5102159;5102168;5102187</t>
         </is>
       </c>
       <c r="L214" t="inlineStr"/>
       <c r="M214" t="inlineStr">
         <is>
-          <t>lines 24 and 30 resolve uniquely to serials 5101936 and 5101943, and 2 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 24 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N214" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 33 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 76 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O214" t="inlineStr">
@@ -13227,7 +13159,7 @@
       <c r="H215" t="inlineStr"/>
       <c r="I215" t="inlineStr">
         <is>
-          <t>ambiguous(4)</t>
+          <t>ambiguous(9)</t>
         </is>
       </c>
       <c r="J215" t="n">
@@ -13235,22 +13167,18 @@
       </c>
       <c r="K215" t="inlineStr">
         <is>
-          <t>5101927;5101940;5102018;5102019</t>
-        </is>
-      </c>
-      <c r="L215" t="inlineStr">
-        <is>
-          <t>5101940</t>
-        </is>
-      </c>
+          <t>5101292;5101334;5101471;5101927;5101940;5102018;5102019;5102025;5102134</t>
+        </is>
+      </c>
+      <c r="L215" t="inlineStr"/>
       <c r="M215" t="inlineStr">
         <is>
-          <t>lines 24 and 30 resolve uniquely to serials 5101936 and 5101943; of this line's 4 candidates exactly one, 5101940, lies in that run at exactly the position an unbroken run would put it</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 2 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N215" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 4 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 9 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O215" t="inlineStr">
@@ -13294,7 +13222,7 @@
       <c r="H216" t="inlineStr"/>
       <c r="I216" t="inlineStr">
         <is>
-          <t>ambiguous(7)</t>
+          <t>ambiguous(4)</t>
         </is>
       </c>
       <c r="J216" t="n">
@@ -13302,22 +13230,18 @@
       </c>
       <c r="K216" t="inlineStr">
         <is>
-          <t>5101258;5101278;5101331;5101425;5101910;5101942;5101983</t>
-        </is>
-      </c>
-      <c r="L216" t="inlineStr">
-        <is>
-          <t>5101942</t>
-        </is>
-      </c>
+          <t>5101306;5101425;5101910;5101913</t>
+        </is>
+      </c>
+      <c r="L216" t="inlineStr"/>
       <c r="M216" t="inlineStr">
         <is>
-          <t>lines 24 and 30 resolve uniquely to serials 5101936 and 5101943; of this line's 7 candidates exactly one, 5101942, lies in that run, and an unbroken run would put this line at 5101941</t>
+          <t>lines 22 and 30 resolve uniquely to serials 5101709 and 5101943, and 2 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
         </is>
       </c>
       <c r="N216" t="inlineStr">
         <is>
-          <t>the fingerprint over 24 columns matches 7 IPUMS households and does not distinguish them; no serial is attached</t>
+          <t>the fingerprint over 24 columns matches 4 IPUMS households and does not distinguish them; no serial is attached</t>
         </is>
       </c>
       <c r="O216" t="inlineStr">

</xml_diff>

<commit_message>
T-0963: the 1840 census printed 212 and 213 read to the name and the cell
</commit_message>
<xml_diff>
--- a/chicago/reference/census1840/validation/T-0504_1840_name_serial_crosswalk.xlsx
+++ b/chicago/reference/census1840/validation/T-0504_1840_name_serial_crosswalk.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O637"/>
+  <dimension ref="A1:O698"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38687,6 +38687,3669 @@
         </is>
       </c>
     </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B638" t="n">
+        <v>213</v>
+      </c>
+      <c r="C638" t="n">
+        <v>1</v>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>Casper [M]uller</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>Casper Muller</t>
+        </is>
+      </c>
+      <c r="F638" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G638" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H638" t="inlineStr"/>
+      <c r="I638" t="inlineStr">
+        <is>
+          <t>ambiguous(10)</t>
+        </is>
+      </c>
+      <c r="J638" t="n">
+        <v>26</v>
+      </c>
+      <c r="K638" t="inlineStr">
+        <is>
+          <t>5101381;5101393;5101398;5101413;5101423;5101446;5101456;5101594;5101595;5101596</t>
+        </is>
+      </c>
+      <c r="L638" t="inlineStr"/>
+      <c r="M638" t="inlineStr"/>
+      <c r="N638" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 10 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O638" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B639" t="n">
+        <v>213</v>
+      </c>
+      <c r="C639" t="n">
+        <v>2</v>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>W[m]. [?] Sh[e]n[e]r</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>William [?] Shener</t>
+        </is>
+      </c>
+      <c r="F639" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G639" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H639" t="inlineStr">
+        <is>
+          <t>5101449</t>
+        </is>
+      </c>
+      <c r="I639" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
+      <c r="J639" t="n">
+        <v>26</v>
+      </c>
+      <c r="K639" t="inlineStr"/>
+      <c r="L639" t="inlineStr"/>
+      <c r="M639" t="inlineStr"/>
+      <c r="N639" t="inlineStr">
+        <is>
+          <t>free-white age-band fingerprint over 26 of the schedule's 26 columns matches exactly one of the 964 IPUMS households</t>
+        </is>
+      </c>
+      <c r="O639" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B640" t="n">
+        <v>213</v>
+      </c>
+      <c r="C640" t="n">
+        <v>3</v>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>[D]. [B]. [F]ischo[f]</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>D. B. Fischof</t>
+        </is>
+      </c>
+      <c r="F640" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G640" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H640" t="inlineStr"/>
+      <c r="I640" t="inlineStr">
+        <is>
+          <t>ambiguous(11)</t>
+        </is>
+      </c>
+      <c r="J640" t="n">
+        <v>26</v>
+      </c>
+      <c r="K640" t="inlineStr">
+        <is>
+          <t>5101362;5101450;5101516;5101580;5101650;5101654;5101655;5101776;5101783;5101857;5101969</t>
+        </is>
+      </c>
+      <c r="L640" t="inlineStr"/>
+      <c r="M640" t="inlineStr"/>
+      <c r="N640" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 11 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O640" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B641" t="n">
+        <v>213</v>
+      </c>
+      <c r="C641" t="n">
+        <v>4</v>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>E[ph]e[a]n [?] Sha[i]l[s]</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>[?] Shails</t>
+        </is>
+      </c>
+      <c r="F641" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G641" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H641" t="inlineStr"/>
+      <c r="I641" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J641" t="n">
+        <v>26</v>
+      </c>
+      <c r="K641" t="inlineStr"/>
+      <c r="L641" t="inlineStr"/>
+      <c r="M641" t="inlineStr"/>
+      <c r="N641" t="inlineStr">
+        <is>
+          <t>no IPUMS household carries this pattern over the 26 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
+        </is>
+      </c>
+      <c r="O641" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B642" t="n">
+        <v>213</v>
+      </c>
+      <c r="C642" t="n">
+        <v>5</v>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>Ch[s]. Raymond</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>Charles Raymond</t>
+        </is>
+      </c>
+      <c r="F642" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G642" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H642" t="inlineStr"/>
+      <c r="I642" t="inlineStr">
+        <is>
+          <t>ambiguous(8)</t>
+        </is>
+      </c>
+      <c r="J642" t="n">
+        <v>26</v>
+      </c>
+      <c r="K642" t="inlineStr">
+        <is>
+          <t>5101416;5101452;5101453;5101498;5101959;5101979;5102032;5102051</t>
+        </is>
+      </c>
+      <c r="L642" t="inlineStr"/>
+      <c r="M642" t="inlineStr"/>
+      <c r="N642" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 8 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O642" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B643" t="n">
+        <v>213</v>
+      </c>
+      <c r="C643" t="n">
+        <v>6</v>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>[N]. B. Ca[r]t[e]r</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>N. B. Carter</t>
+        </is>
+      </c>
+      <c r="F643" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G643" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H643" t="inlineStr"/>
+      <c r="I643" t="inlineStr">
+        <is>
+          <t>ambiguous(8)</t>
+        </is>
+      </c>
+      <c r="J643" t="n">
+        <v>26</v>
+      </c>
+      <c r="K643" t="inlineStr">
+        <is>
+          <t>5101416;5101452;5101453;5101498;5101959;5101979;5102032;5102051</t>
+        </is>
+      </c>
+      <c r="L643" t="inlineStr"/>
+      <c r="M643" t="inlineStr"/>
+      <c r="N643" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 8 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O643" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B644" t="n">
+        <v>213</v>
+      </c>
+      <c r="C644" t="n">
+        <v>7</v>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>Nath[a]n [E]. King</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>Nathan E. King</t>
+        </is>
+      </c>
+      <c r="F644" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G644" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H644" t="inlineStr"/>
+      <c r="I644" t="inlineStr">
+        <is>
+          <t>ambiguous(43)</t>
+        </is>
+      </c>
+      <c r="J644" t="n">
+        <v>26</v>
+      </c>
+      <c r="K644" t="inlineStr">
+        <is>
+          <t>5101373;5101374;5101375;5101376;5101378;5101401;5101402;5101403;5101406;5101419;5101421;5101433;5101454;5101458;5101460;5101469;5101494;5101499;5101500;5101501;5101508;5101511;5101513;5101518;5101523;5101524;5101558;5101587;5101590;5101598;5101600;5101612;5101613;5101622;5101623;5101633;5101637;5101646;5101676;5101746;5102034;5102173;5102174</t>
+        </is>
+      </c>
+      <c r="L644" t="inlineStr"/>
+      <c r="M644" t="inlineStr"/>
+      <c r="N644" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 43 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O644" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B645" t="n">
+        <v>213</v>
+      </c>
+      <c r="C645" t="n">
+        <v>8</v>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>[Ch]ad[w]ell &amp; H. Vail</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>Chadwell &amp; H. Vail</t>
+        </is>
+      </c>
+      <c r="F645" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G645" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H645" t="inlineStr"/>
+      <c r="I645" t="inlineStr">
+        <is>
+          <t>ambiguous(6)</t>
+        </is>
+      </c>
+      <c r="J645" t="n">
+        <v>26</v>
+      </c>
+      <c r="K645" t="inlineStr">
+        <is>
+          <t>5101417;5101455;5101610;5102008;5102024;5102179</t>
+        </is>
+      </c>
+      <c r="L645" t="inlineStr"/>
+      <c r="M645" t="inlineStr"/>
+      <c r="N645" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 6 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O645" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B646" t="n">
+        <v>213</v>
+      </c>
+      <c r="C646" t="n">
+        <v>9</v>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>[S]. M. Wag[e]r</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>S. M. Wager</t>
+        </is>
+      </c>
+      <c r="F646" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G646" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H646" t="inlineStr"/>
+      <c r="I646" t="inlineStr">
+        <is>
+          <t>ambiguous(10)</t>
+        </is>
+      </c>
+      <c r="J646" t="n">
+        <v>26</v>
+      </c>
+      <c r="K646" t="inlineStr">
+        <is>
+          <t>5101381;5101393;5101398;5101413;5101423;5101446;5101456;5101594;5101595;5101596</t>
+        </is>
+      </c>
+      <c r="L646" t="inlineStr"/>
+      <c r="M646" t="inlineStr"/>
+      <c r="N646" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 10 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O646" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B647" t="n">
+        <v>213</v>
+      </c>
+      <c r="C647" t="n">
+        <v>10</v>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>[?] W[m]. C[l]on[e]</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>[?] William Clone</t>
+        </is>
+      </c>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G647" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H647" t="inlineStr"/>
+      <c r="I647" t="inlineStr">
+        <is>
+          <t>ambiguous(3)</t>
+        </is>
+      </c>
+      <c r="J647" t="n">
+        <v>26</v>
+      </c>
+      <c r="K647" t="inlineStr">
+        <is>
+          <t>5101420;5101457;5101810</t>
+        </is>
+      </c>
+      <c r="L647" t="inlineStr"/>
+      <c r="M647" t="inlineStr"/>
+      <c r="N647" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 3 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O647" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B648" t="n">
+        <v>213</v>
+      </c>
+      <c r="C648" t="n">
+        <v>11</v>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>[A]. [N]. Dea[r]d[e]n</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>A. N. Dearden</t>
+        </is>
+      </c>
+      <c r="F648" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G648" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H648" t="inlineStr"/>
+      <c r="I648" t="inlineStr">
+        <is>
+          <t>ambiguous(43)</t>
+        </is>
+      </c>
+      <c r="J648" t="n">
+        <v>26</v>
+      </c>
+      <c r="K648" t="inlineStr">
+        <is>
+          <t>5101373;5101374;5101375;5101376;5101378;5101401;5101402;5101403;5101406;5101419;5101421;5101433;5101454;5101458;5101460;5101469;5101494;5101499;5101500;5101501;5101508;5101511;5101513;5101518;5101523;5101524;5101558;5101587;5101590;5101598;5101600;5101612;5101613;5101622;5101623;5101633;5101637;5101646;5101676;5101746;5102034;5102173;5102174</t>
+        </is>
+      </c>
+      <c r="L648" t="inlineStr"/>
+      <c r="M648" t="inlineStr"/>
+      <c r="N648" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 43 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O648" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B649" t="n">
+        <v>213</v>
+      </c>
+      <c r="C649" t="n">
+        <v>12</v>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>[E]. [K]. [?]</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>[?]</t>
+        </is>
+      </c>
+      <c r="F649" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G649" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H649" t="inlineStr"/>
+      <c r="I649" t="inlineStr">
+        <is>
+          <t>ambiguous(3)</t>
+        </is>
+      </c>
+      <c r="J649" t="n">
+        <v>26</v>
+      </c>
+      <c r="K649" t="inlineStr">
+        <is>
+          <t>5101408;5101409;5101459</t>
+        </is>
+      </c>
+      <c r="L649" t="inlineStr"/>
+      <c r="M649" t="inlineStr"/>
+      <c r="N649" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 3 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O649" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B650" t="n">
+        <v>213</v>
+      </c>
+      <c r="C650" t="n">
+        <v>13</v>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>[H]. [H]. Ryan</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>H. H. Ryan</t>
+        </is>
+      </c>
+      <c r="F650" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G650" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H650" t="inlineStr"/>
+      <c r="I650" t="inlineStr">
+        <is>
+          <t>ambiguous(43)</t>
+        </is>
+      </c>
+      <c r="J650" t="n">
+        <v>26</v>
+      </c>
+      <c r="K650" t="inlineStr">
+        <is>
+          <t>5101373;5101374;5101375;5101376;5101378;5101401;5101402;5101403;5101406;5101419;5101421;5101433;5101454;5101458;5101460;5101469;5101494;5101499;5101500;5101501;5101508;5101511;5101513;5101518;5101523;5101524;5101558;5101587;5101590;5101598;5101600;5101612;5101613;5101622;5101623;5101633;5101637;5101646;5101676;5101746;5102034;5102173;5102174</t>
+        </is>
+      </c>
+      <c r="L650" t="inlineStr"/>
+      <c r="M650" t="inlineStr"/>
+      <c r="N650" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 43 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O650" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B651" t="n">
+        <v>213</v>
+      </c>
+      <c r="C651" t="n">
+        <v>14</v>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>Chaunc[y] [S]hell</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>Chauncy Shell</t>
+        </is>
+      </c>
+      <c r="F651" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G651" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H651" t="inlineStr"/>
+      <c r="I651" t="inlineStr">
+        <is>
+          <t>ambiguous(2)</t>
+        </is>
+      </c>
+      <c r="J651" t="n">
+        <v>26</v>
+      </c>
+      <c r="K651" t="inlineStr">
+        <is>
+          <t>5101451;5101461</t>
+        </is>
+      </c>
+      <c r="L651" t="inlineStr"/>
+      <c r="M651" t="inlineStr"/>
+      <c r="N651" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 2 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O651" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B652" t="n">
+        <v>213</v>
+      </c>
+      <c r="C652" t="n">
+        <v>15</v>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>[Jos]. Pat[h]</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>Jos. Path</t>
+        </is>
+      </c>
+      <c r="F652" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G652" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H652" t="inlineStr"/>
+      <c r="I652" t="inlineStr">
+        <is>
+          <t>ambiguous(10)</t>
+        </is>
+      </c>
+      <c r="J652" t="n">
+        <v>26</v>
+      </c>
+      <c r="K652" t="inlineStr">
+        <is>
+          <t>5101266;5101418;5101462;5101512;5101640;5101645;5101664;5101751;5101960;5102190</t>
+        </is>
+      </c>
+      <c r="L652" t="inlineStr"/>
+      <c r="M652" t="inlineStr"/>
+      <c r="N652" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 10 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O652" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B653" t="n">
+        <v>213</v>
+      </c>
+      <c r="C653" t="n">
+        <v>16</v>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>[?]. [B]. Ba[?]</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>[?]</t>
+        </is>
+      </c>
+      <c r="F653" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G653" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H653" t="inlineStr"/>
+      <c r="I653" t="inlineStr">
+        <is>
+          <t>ambiguous(3)</t>
+        </is>
+      </c>
+      <c r="J653" t="n">
+        <v>26</v>
+      </c>
+      <c r="K653" t="inlineStr">
+        <is>
+          <t>5101290;5101463;5102140</t>
+        </is>
+      </c>
+      <c r="L653" t="inlineStr"/>
+      <c r="M653" t="inlineStr"/>
+      <c r="N653" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 3 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O653" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B654" t="n">
+        <v>213</v>
+      </c>
+      <c r="C654" t="n">
+        <v>17</v>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>Robert [F]ol[g]an</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>Robert Folgan</t>
+        </is>
+      </c>
+      <c r="F654" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G654" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H654" t="inlineStr"/>
+      <c r="I654" t="inlineStr">
+        <is>
+          <t>ambiguous(43)</t>
+        </is>
+      </c>
+      <c r="J654" t="n">
+        <v>26</v>
+      </c>
+      <c r="K654" t="inlineStr">
+        <is>
+          <t>5101273;5101291;5101294;5101321;5101324;5101337;5101432;5101434;5101443;5101464;5101476;5101479;5101485;5101551;5101552;5101606;5101631;5101656;5101678;5101739;5101743;5101759;5101765;5101812;5101820;5101822;5101853;5101880;5101882;5101883;5101906;5101918;5101928;5101947;5101954;5101956;5101985;5101990;5102050;5102155;5102156;5102159;5102168</t>
+        </is>
+      </c>
+      <c r="L654" t="inlineStr"/>
+      <c r="M654" t="inlineStr"/>
+      <c r="N654" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 43 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O654" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B655" t="n">
+        <v>213</v>
+      </c>
+      <c r="C655" t="n">
+        <v>18</v>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>[W]m. Ra[n]kin</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>William Rankin</t>
+        </is>
+      </c>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G655" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H655" t="inlineStr">
+        <is>
+          <t>5101435</t>
+        </is>
+      </c>
+      <c r="I655" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
+      <c r="J655" t="n">
+        <v>26</v>
+      </c>
+      <c r="K655" t="inlineStr"/>
+      <c r="L655" t="inlineStr"/>
+      <c r="M655" t="inlineStr"/>
+      <c r="N655" t="inlineStr">
+        <is>
+          <t>free-white age-band fingerprint over 26 of the schedule's 26 columns matches exactly one of the 964 IPUMS households</t>
+        </is>
+      </c>
+      <c r="O655" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B656" t="n">
+        <v>213</v>
+      </c>
+      <c r="C656" t="n">
+        <v>19</v>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>[?] A[b]e[l]e[s]</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>[?] Abeles</t>
+        </is>
+      </c>
+      <c r="F656" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G656" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H656" t="inlineStr">
+        <is>
+          <t>5101436</t>
+        </is>
+      </c>
+      <c r="I656" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
+      <c r="J656" t="n">
+        <v>26</v>
+      </c>
+      <c r="K656" t="inlineStr"/>
+      <c r="L656" t="inlineStr"/>
+      <c r="M656" t="inlineStr"/>
+      <c r="N656" t="inlineStr">
+        <is>
+          <t>free-white age-band fingerprint over 26 of the schedule's 26 columns matches exactly one of the 964 IPUMS households</t>
+        </is>
+      </c>
+      <c r="O656" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B657" t="n">
+        <v>213</v>
+      </c>
+      <c r="C657" t="n">
+        <v>20</v>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>[W]. [H]o[d]son</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>W. Hodson</t>
+        </is>
+      </c>
+      <c r="F657" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G657" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H657" t="inlineStr">
+        <is>
+          <t>5101437</t>
+        </is>
+      </c>
+      <c r="I657" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
+      <c r="J657" t="n">
+        <v>26</v>
+      </c>
+      <c r="K657" t="inlineStr"/>
+      <c r="L657" t="inlineStr"/>
+      <c r="M657" t="inlineStr"/>
+      <c r="N657" t="inlineStr">
+        <is>
+          <t>free-white age-band fingerprint over 26 of the schedule's 26 columns matches exactly one of the 964 IPUMS households</t>
+        </is>
+      </c>
+      <c r="O657" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B658" t="n">
+        <v>213</v>
+      </c>
+      <c r="C658" t="n">
+        <v>21</v>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>[H]. [Sp]a[rk]e[r]</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>H. Sparker</t>
+        </is>
+      </c>
+      <c r="F658" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G658" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H658" t="inlineStr">
+        <is>
+          <t>5101438</t>
+        </is>
+      </c>
+      <c r="I658" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
+      <c r="J658" t="n">
+        <v>26</v>
+      </c>
+      <c r="K658" t="inlineStr"/>
+      <c r="L658" t="inlineStr"/>
+      <c r="M658" t="inlineStr"/>
+      <c r="N658" t="inlineStr">
+        <is>
+          <t>free-white age-band fingerprint over 26 of the schedule's 26 columns matches exactly one of the 964 IPUMS households</t>
+        </is>
+      </c>
+      <c r="O658" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B659" t="n">
+        <v>213</v>
+      </c>
+      <c r="C659" t="n">
+        <v>22</v>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>John H[e]in[i]ck</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>John Heinick</t>
+        </is>
+      </c>
+      <c r="F659" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G659" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H659" t="inlineStr">
+        <is>
+          <t>5101439</t>
+        </is>
+      </c>
+      <c r="I659" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
+      <c r="J659" t="n">
+        <v>26</v>
+      </c>
+      <c r="K659" t="inlineStr"/>
+      <c r="L659" t="inlineStr"/>
+      <c r="M659" t="inlineStr"/>
+      <c r="N659" t="inlineStr">
+        <is>
+          <t>free-white age-band fingerprint over 26 of the schedule's 26 columns matches exactly one of the 964 IPUMS households</t>
+        </is>
+      </c>
+      <c r="O659" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B660" t="n">
+        <v>213</v>
+      </c>
+      <c r="C660" t="n">
+        <v>23</v>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>[Jos]. Whit[a]k[e]r</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>Jos. Whitaker</t>
+        </is>
+      </c>
+      <c r="F660" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G660" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H660" t="inlineStr"/>
+      <c r="I660" t="inlineStr">
+        <is>
+          <t>ambiguous(6)</t>
+        </is>
+      </c>
+      <c r="J660" t="n">
+        <v>26</v>
+      </c>
+      <c r="K660" t="inlineStr">
+        <is>
+          <t>5101440;5101728;5101852;5102005;5102094;5102157</t>
+        </is>
+      </c>
+      <c r="L660" t="inlineStr">
+        <is>
+          <t>5101440</t>
+        </is>
+      </c>
+      <c r="M660" t="inlineStr">
+        <is>
+          <t>lines 22 and 24 resolve uniquely to serials 5101439 and 5101441; of this line's 6 candidates exactly one, 5101440, lies in that run at exactly the position an unbroken run would put it</t>
+        </is>
+      </c>
+      <c r="N660" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 6 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O660" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B661" t="n">
+        <v>213</v>
+      </c>
+      <c r="C661" t="n">
+        <v>24</v>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>John Rogan</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>John Rogan</t>
+        </is>
+      </c>
+      <c r="F661" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G661" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H661" t="inlineStr">
+        <is>
+          <t>5101441</t>
+        </is>
+      </c>
+      <c r="I661" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
+      <c r="J661" t="n">
+        <v>26</v>
+      </c>
+      <c r="K661" t="inlineStr"/>
+      <c r="L661" t="inlineStr"/>
+      <c r="M661" t="inlineStr"/>
+      <c r="N661" t="inlineStr">
+        <is>
+          <t>free-white age-band fingerprint over 26 of the schedule's 26 columns matches exactly one of the 964 IPUMS households</t>
+        </is>
+      </c>
+      <c r="O661" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B662" t="n">
+        <v>213</v>
+      </c>
+      <c r="C662" t="n">
+        <v>25</v>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>A. [S]. Benne[t]</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>A. S. Bennet</t>
+        </is>
+      </c>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G662" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H662" t="inlineStr"/>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>ambiguous(2)</t>
+        </is>
+      </c>
+      <c r="J662" t="n">
+        <v>26</v>
+      </c>
+      <c r="K662" t="inlineStr">
+        <is>
+          <t>5101442;5102092</t>
+        </is>
+      </c>
+      <c r="L662" t="inlineStr">
+        <is>
+          <t>5101442</t>
+        </is>
+      </c>
+      <c r="M662" t="inlineStr">
+        <is>
+          <t>lines 24 and 27 resolve uniquely to serials 5101441 and 5101444; of this line's 2 candidates exactly one, 5101442, lies in that run at exactly the position an unbroken run would put it</t>
+        </is>
+      </c>
+      <c r="N662" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 2 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O662" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B663" t="n">
+        <v>213</v>
+      </c>
+      <c r="C663" t="n">
+        <v>26</v>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>Th[os]. P[ag]e</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>Thomas Page</t>
+        </is>
+      </c>
+      <c r="F663" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G663" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H663" t="inlineStr"/>
+      <c r="I663" t="inlineStr">
+        <is>
+          <t>ambiguous(43)</t>
+        </is>
+      </c>
+      <c r="J663" t="n">
+        <v>26</v>
+      </c>
+      <c r="K663" t="inlineStr">
+        <is>
+          <t>5101273;5101291;5101294;5101321;5101324;5101337;5101432;5101434;5101443;5101464;5101476;5101479;5101485;5101551;5101552;5101606;5101631;5101656;5101678;5101739;5101743;5101759;5101765;5101812;5101820;5101822;5101853;5101880;5101882;5101883;5101906;5101918;5101928;5101947;5101954;5101956;5101985;5101990;5102050;5102155;5102156;5102159;5102168</t>
+        </is>
+      </c>
+      <c r="L663" t="inlineStr">
+        <is>
+          <t>5101443</t>
+        </is>
+      </c>
+      <c r="M663" t="inlineStr">
+        <is>
+          <t>lines 24 and 27 resolve uniquely to serials 5101441 and 5101444; of this line's 43 candidates exactly one, 5101443, lies in that run at exactly the position an unbroken run would put it</t>
+        </is>
+      </c>
+      <c r="N663" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 43 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O663" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B664" t="n">
+        <v>213</v>
+      </c>
+      <c r="C664" t="n">
+        <v>27</v>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>[Ja]s. M[c]Lea[n]</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>James McLean</t>
+        </is>
+      </c>
+      <c r="F664" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G664" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H664" t="inlineStr">
+        <is>
+          <t>5101444</t>
+        </is>
+      </c>
+      <c r="I664" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
+      <c r="J664" t="n">
+        <v>26</v>
+      </c>
+      <c r="K664" t="inlineStr"/>
+      <c r="L664" t="inlineStr"/>
+      <c r="M664" t="inlineStr"/>
+      <c r="N664" t="inlineStr">
+        <is>
+          <t>free-white age-band fingerprint over 26 of the schedule's 26 columns matches exactly one of the 964 IPUMS households</t>
+        </is>
+      </c>
+      <c r="O664" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B665" t="n">
+        <v>213</v>
+      </c>
+      <c r="C665" t="n">
+        <v>28</v>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>[L]. [A]. [R]a[ll]s[t]one</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>L. A. Rallstone</t>
+        </is>
+      </c>
+      <c r="F665" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G665" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H665" t="inlineStr"/>
+      <c r="I665" t="inlineStr">
+        <is>
+          <t>ambiguous(6)</t>
+        </is>
+      </c>
+      <c r="J665" t="n">
+        <v>26</v>
+      </c>
+      <c r="K665" t="inlineStr">
+        <is>
+          <t>5101283;5101392;5101445;5101559;5101696;5101863</t>
+        </is>
+      </c>
+      <c r="L665" t="inlineStr">
+        <is>
+          <t>5101445</t>
+        </is>
+      </c>
+      <c r="M665" t="inlineStr">
+        <is>
+          <t>lines 27 and 30 resolve uniquely to serials 5101444 and 5101448; of this line's 6 candidates exactly one, 5101445, lies in that run at exactly the position an unbroken run would put it</t>
+        </is>
+      </c>
+      <c r="N665" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 6 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O665" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B666" t="n">
+        <v>213</v>
+      </c>
+      <c r="C666" t="n">
+        <v>29</v>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>M. [H]. Magi[e]</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>M. H. Magie</t>
+        </is>
+      </c>
+      <c r="F666" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G666" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H666" t="inlineStr"/>
+      <c r="I666" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J666" t="n">
+        <v>26</v>
+      </c>
+      <c r="K666" t="inlineStr"/>
+      <c r="L666" t="inlineStr"/>
+      <c r="M666" t="inlineStr"/>
+      <c r="N666" t="inlineStr">
+        <is>
+          <t>no IPUMS household carries this pattern over the 26 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
+        </is>
+      </c>
+      <c r="O666" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RK</t>
+        </is>
+      </c>
+      <c r="B667" t="n">
+        <v>213</v>
+      </c>
+      <c r="C667" t="n">
+        <v>30</v>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>[F]. C. Sherman</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>F. C. Sherman</t>
+        </is>
+      </c>
+      <c r="F667" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G667" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H667" t="inlineStr">
+        <is>
+          <t>5101448</t>
+        </is>
+      </c>
+      <c r="I667" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
+      <c r="J667" t="n">
+        <v>26</v>
+      </c>
+      <c r="K667" t="inlineStr"/>
+      <c r="L667" t="inlineStr"/>
+      <c r="M667" t="inlineStr"/>
+      <c r="N667" t="inlineStr">
+        <is>
+          <t>free-white age-band fingerprint over 26 of the schedule's 26 columns matches exactly one of the 964 IPUMS households</t>
+        </is>
+      </c>
+      <c r="O667" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RK.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B668" t="n">
+        <v>212</v>
+      </c>
+      <c r="C668" t="n">
+        <v>1</v>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>[?] Sawyer</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>[?] Sawyer</t>
+        </is>
+      </c>
+      <c r="F668" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G668" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H668" t="inlineStr"/>
+      <c r="I668" t="inlineStr">
+        <is>
+          <t>ambiguous(8)</t>
+        </is>
+      </c>
+      <c r="J668" t="n">
+        <v>26</v>
+      </c>
+      <c r="K668" t="inlineStr">
+        <is>
+          <t>5101416;5101452;5101453;5101498;5101959;5101979;5102032;5102051</t>
+        </is>
+      </c>
+      <c r="L668" t="inlineStr"/>
+      <c r="M668" t="inlineStr"/>
+      <c r="N668" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 8 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O668" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B669" t="n">
+        <v>212</v>
+      </c>
+      <c r="C669" t="n">
+        <v>2</v>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>Joseph Shields</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>Joseph Shields</t>
+        </is>
+      </c>
+      <c r="F669" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G669" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H669" t="inlineStr"/>
+      <c r="I669" t="inlineStr">
+        <is>
+          <t>ambiguous(3)</t>
+        </is>
+      </c>
+      <c r="J669" t="n">
+        <v>26</v>
+      </c>
+      <c r="K669" t="inlineStr">
+        <is>
+          <t>5101420;5101457;5101810</t>
+        </is>
+      </c>
+      <c r="L669" t="inlineStr"/>
+      <c r="M669" t="inlineStr"/>
+      <c r="N669" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 3 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O669" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B670" t="n">
+        <v>212</v>
+      </c>
+      <c r="C670" t="n">
+        <v>3</v>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>And[e]rson [L]. Co[x]</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>Anderson L. Cox</t>
+        </is>
+      </c>
+      <c r="F670" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G670" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H670" t="inlineStr"/>
+      <c r="I670" t="inlineStr">
+        <is>
+          <t>ambiguous(43)</t>
+        </is>
+      </c>
+      <c r="J670" t="n">
+        <v>26</v>
+      </c>
+      <c r="K670" t="inlineStr">
+        <is>
+          <t>5101373;5101374;5101375;5101376;5101378;5101401;5101402;5101403;5101406;5101419;5101421;5101433;5101454;5101458;5101460;5101469;5101494;5101499;5101500;5101501;5101508;5101511;5101513;5101518;5101523;5101524;5101558;5101587;5101590;5101598;5101600;5101612;5101613;5101622;5101623;5101633;5101637;5101646;5101676;5101746;5102034;5102173;5102174</t>
+        </is>
+      </c>
+      <c r="L670" t="inlineStr"/>
+      <c r="M670" t="inlineStr"/>
+      <c r="N670" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 43 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O670" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B671" t="n">
+        <v>212</v>
+      </c>
+      <c r="C671" t="n">
+        <v>4</v>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>Robert Ba[d]y</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>Robert Bady</t>
+        </is>
+      </c>
+      <c r="F671" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G671" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H671" t="inlineStr">
+        <is>
+          <t>5101422</t>
+        </is>
+      </c>
+      <c r="I671" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
+      <c r="J671" t="n">
+        <v>26</v>
+      </c>
+      <c r="K671" t="inlineStr"/>
+      <c r="L671" t="inlineStr"/>
+      <c r="M671" t="inlineStr"/>
+      <c r="N671" t="inlineStr">
+        <is>
+          <t>free-white age-band fingerprint over 26 of the schedule's 26 columns matches exactly one of the 964 IPUMS households</t>
+        </is>
+      </c>
+      <c r="O671" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B672" t="n">
+        <v>212</v>
+      </c>
+      <c r="C672" t="n">
+        <v>5</v>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>D. H. [?]anda[c]k</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>D. H. [?]</t>
+        </is>
+      </c>
+      <c r="F672" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G672" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H672" t="inlineStr"/>
+      <c r="I672" t="inlineStr">
+        <is>
+          <t>ambiguous(10)</t>
+        </is>
+      </c>
+      <c r="J672" t="n">
+        <v>26</v>
+      </c>
+      <c r="K672" t="inlineStr">
+        <is>
+          <t>5101381;5101393;5101398;5101413;5101423;5101446;5101456;5101594;5101595;5101596</t>
+        </is>
+      </c>
+      <c r="L672" t="inlineStr">
+        <is>
+          <t>5101423</t>
+        </is>
+      </c>
+      <c r="M672" t="inlineStr">
+        <is>
+          <t>lines 4 and 6 resolve uniquely to serials 5101422 and 5101424; of this line's 10 candidates exactly one, 5101423, lies in that run at exactly the position an unbroken run would put it</t>
+        </is>
+      </c>
+      <c r="N672" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 10 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O672" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B673" t="n">
+        <v>212</v>
+      </c>
+      <c r="C673" t="n">
+        <v>6</v>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>Marg[u]erite M[e]rra[r]d</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>Marguerite Merrard</t>
+        </is>
+      </c>
+      <c r="F673" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G673" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H673" t="inlineStr">
+        <is>
+          <t>5101424</t>
+        </is>
+      </c>
+      <c r="I673" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
+      <c r="J673" t="n">
+        <v>26</v>
+      </c>
+      <c r="K673" t="inlineStr"/>
+      <c r="L673" t="inlineStr"/>
+      <c r="M673" t="inlineStr"/>
+      <c r="N673" t="inlineStr">
+        <is>
+          <t>free-white age-band fingerprint over 26 of the schedule's 26 columns matches exactly one of the 964 IPUMS households</t>
+        </is>
+      </c>
+      <c r="O673" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B674" t="n">
+        <v>212</v>
+      </c>
+      <c r="C674" t="n">
+        <v>7</v>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>David Bra[m]elin</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>David Bramelin</t>
+        </is>
+      </c>
+      <c r="F674" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G674" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H674" t="inlineStr"/>
+      <c r="I674" t="inlineStr">
+        <is>
+          <t>ambiguous(2)</t>
+        </is>
+      </c>
+      <c r="J674" t="n">
+        <v>26</v>
+      </c>
+      <c r="K674" t="inlineStr">
+        <is>
+          <t>5101425;5101910</t>
+        </is>
+      </c>
+      <c r="L674" t="inlineStr">
+        <is>
+          <t>5101425</t>
+        </is>
+      </c>
+      <c r="M674" t="inlineStr">
+        <is>
+          <t>lines 6 and 8 resolve uniquely to serials 5101424 and 5101426; of this line's 2 candidates exactly one, 5101425, lies in that run at exactly the position an unbroken run would put it</t>
+        </is>
+      </c>
+      <c r="N674" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 2 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O674" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B675" t="n">
+        <v>212</v>
+      </c>
+      <c r="C675" t="n">
+        <v>8</v>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>Robt. Watts</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>Robert Watts</t>
+        </is>
+      </c>
+      <c r="F675" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G675" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H675" t="inlineStr">
+        <is>
+          <t>5101426</t>
+        </is>
+      </c>
+      <c r="I675" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
+      <c r="J675" t="n">
+        <v>26</v>
+      </c>
+      <c r="K675" t="inlineStr"/>
+      <c r="L675" t="inlineStr"/>
+      <c r="M675" t="inlineStr"/>
+      <c r="N675" t="inlineStr">
+        <is>
+          <t>free-white age-band fingerprint over 26 of the schedule's 26 columns matches exactly one of the 964 IPUMS households</t>
+        </is>
+      </c>
+      <c r="O675" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B676" t="n">
+        <v>212</v>
+      </c>
+      <c r="C676" t="n">
+        <v>9</v>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>Wm. Raymond</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>William Raymond</t>
+        </is>
+      </c>
+      <c r="F676" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G676" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H676" t="inlineStr"/>
+      <c r="I676" t="inlineStr">
+        <is>
+          <t>ambiguous(18)</t>
+        </is>
+      </c>
+      <c r="J676" t="n">
+        <v>26</v>
+      </c>
+      <c r="K676" t="inlineStr">
+        <is>
+          <t>5101427;5101555;5101557;5101653;5101682;5101722;5101827;5101864;5101869;5101890;5101905;5101939;5101973;5102000;5102011;5102052;5102105;5102144</t>
+        </is>
+      </c>
+      <c r="L676" t="inlineStr">
+        <is>
+          <t>5101427</t>
+        </is>
+      </c>
+      <c r="M676" t="inlineStr">
+        <is>
+          <t>lines 8 and 10 resolve uniquely to serials 5101426 and 5101428; of this line's 18 candidates exactly one, 5101427, lies in that run at exactly the position an unbroken run would put it</t>
+        </is>
+      </c>
+      <c r="N676" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 18 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O676" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B677" t="n">
+        <v>212</v>
+      </c>
+      <c r="C677" t="n">
+        <v>10</v>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>W[m]. [W]arner</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>William Warner</t>
+        </is>
+      </c>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G677" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H677" t="inlineStr">
+        <is>
+          <t>5101428</t>
+        </is>
+      </c>
+      <c r="I677" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
+      <c r="J677" t="n">
+        <v>26</v>
+      </c>
+      <c r="K677" t="inlineStr"/>
+      <c r="L677" t="inlineStr"/>
+      <c r="M677" t="inlineStr"/>
+      <c r="N677" t="inlineStr">
+        <is>
+          <t>free-white age-band fingerprint over 26 of the schedule's 26 columns matches exactly one of the 964 IPUMS households</t>
+        </is>
+      </c>
+      <c r="O677" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B678" t="n">
+        <v>212</v>
+      </c>
+      <c r="C678" t="n">
+        <v>11</v>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>Ja[s]. C. [?]</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>Jas. C. [?]</t>
+        </is>
+      </c>
+      <c r="F678" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G678" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H678" t="inlineStr">
+        <is>
+          <t>5101429</t>
+        </is>
+      </c>
+      <c r="I678" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
+      <c r="J678" t="n">
+        <v>26</v>
+      </c>
+      <c r="K678" t="inlineStr"/>
+      <c r="L678" t="inlineStr"/>
+      <c r="M678" t="inlineStr"/>
+      <c r="N678" t="inlineStr">
+        <is>
+          <t>free-white age-band fingerprint over 26 of the schedule's 26 columns matches exactly one of the 964 IPUMS households</t>
+        </is>
+      </c>
+      <c r="O678" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B679" t="n">
+        <v>212</v>
+      </c>
+      <c r="C679" t="n">
+        <v>12</v>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>[?] H. Sherm[an]</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>[?] H. Sherman</t>
+        </is>
+      </c>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G679" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H679" t="inlineStr">
+        <is>
+          <t>5101430</t>
+        </is>
+      </c>
+      <c r="I679" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
+      <c r="J679" t="n">
+        <v>26</v>
+      </c>
+      <c r="K679" t="inlineStr"/>
+      <c r="L679" t="inlineStr"/>
+      <c r="M679" t="inlineStr"/>
+      <c r="N679" t="inlineStr">
+        <is>
+          <t>free-white age-band fingerprint over 26 of the schedule's 26 columns matches exactly one of the 964 IPUMS households</t>
+        </is>
+      </c>
+      <c r="O679" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B680" t="n">
+        <v>212</v>
+      </c>
+      <c r="C680" t="n">
+        <v>13</v>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>[?]. [K]. Bul[l]</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>[?] K. Bull</t>
+        </is>
+      </c>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G680" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H680" t="inlineStr"/>
+      <c r="I680" t="inlineStr">
+        <is>
+          <t>ambiguous(12)</t>
+        </is>
+      </c>
+      <c r="J680" t="n">
+        <v>26</v>
+      </c>
+      <c r="K680" t="inlineStr">
+        <is>
+          <t>5101396;5101397;5101431;5101507;5101548;5101625;5101706;5101724;5101742;5101938;5102036;5102074</t>
+        </is>
+      </c>
+      <c r="L680" t="inlineStr"/>
+      <c r="M680" t="inlineStr"/>
+      <c r="N680" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 12 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O680" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B681" t="n">
+        <v>212</v>
+      </c>
+      <c r="C681" t="n">
+        <v>14</v>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>John Davis</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>John Davis</t>
+        </is>
+      </c>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G681" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H681" t="inlineStr"/>
+      <c r="I681" t="inlineStr">
+        <is>
+          <t>ambiguous(43)</t>
+        </is>
+      </c>
+      <c r="J681" t="n">
+        <v>26</v>
+      </c>
+      <c r="K681" t="inlineStr">
+        <is>
+          <t>5101273;5101291;5101294;5101321;5101324;5101337;5101432;5101434;5101443;5101464;5101476;5101479;5101485;5101551;5101552;5101606;5101631;5101656;5101678;5101739;5101743;5101759;5101765;5101812;5101820;5101822;5101853;5101880;5101882;5101883;5101906;5101918;5101928;5101947;5101954;5101956;5101985;5101990;5102050;5102155;5102156;5102159;5102168</t>
+        </is>
+      </c>
+      <c r="L681" t="inlineStr"/>
+      <c r="M681" t="inlineStr"/>
+      <c r="N681" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 43 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O681" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B682" t="n">
+        <v>212</v>
+      </c>
+      <c r="C682" t="n">
+        <v>15</v>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>Isaac [?] W[il]mo[t]h</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>Isaac [?] Wilmoth</t>
+        </is>
+      </c>
+      <c r="F682" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G682" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H682" t="inlineStr"/>
+      <c r="I682" t="inlineStr">
+        <is>
+          <t>ambiguous(43)</t>
+        </is>
+      </c>
+      <c r="J682" t="n">
+        <v>26</v>
+      </c>
+      <c r="K682" t="inlineStr">
+        <is>
+          <t>5101373;5101374;5101375;5101376;5101378;5101401;5101402;5101403;5101406;5101419;5101421;5101433;5101454;5101458;5101460;5101469;5101494;5101499;5101500;5101501;5101508;5101511;5101513;5101518;5101523;5101524;5101558;5101587;5101590;5101598;5101600;5101612;5101613;5101622;5101623;5101633;5101637;5101646;5101676;5101746;5102034;5102173;5102174</t>
+        </is>
+      </c>
+      <c r="L682" t="inlineStr"/>
+      <c r="M682" t="inlineStr"/>
+      <c r="N682" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 43 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O682" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B683" t="n">
+        <v>212</v>
+      </c>
+      <c r="C683" t="n">
+        <v>16</v>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>Mary Willard</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>Mary Willard</t>
+        </is>
+      </c>
+      <c r="F683" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G683" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H683" t="inlineStr"/>
+      <c r="I683" t="inlineStr">
+        <is>
+          <t>ambiguous(43)</t>
+        </is>
+      </c>
+      <c r="J683" t="n">
+        <v>26</v>
+      </c>
+      <c r="K683" t="inlineStr">
+        <is>
+          <t>5101373;5101374;5101375;5101376;5101378;5101401;5101402;5101403;5101406;5101419;5101421;5101433;5101454;5101458;5101460;5101469;5101494;5101499;5101500;5101501;5101508;5101511;5101513;5101518;5101523;5101524;5101558;5101587;5101590;5101598;5101600;5101612;5101613;5101622;5101623;5101633;5101637;5101646;5101676;5101746;5102034;5102173;5102174</t>
+        </is>
+      </c>
+      <c r="L683" t="inlineStr"/>
+      <c r="M683" t="inlineStr"/>
+      <c r="N683" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 43 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O683" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B684" t="n">
+        <v>212</v>
+      </c>
+      <c r="C684" t="n">
+        <v>17</v>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>Martin Stewart</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>Martin Stewart</t>
+        </is>
+      </c>
+      <c r="F684" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G684" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H684" t="inlineStr">
+        <is>
+          <t>5101404</t>
+        </is>
+      </c>
+      <c r="I684" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
+      <c r="J684" t="n">
+        <v>26</v>
+      </c>
+      <c r="K684" t="inlineStr"/>
+      <c r="L684" t="inlineStr"/>
+      <c r="M684" t="inlineStr"/>
+      <c r="N684" t="inlineStr">
+        <is>
+          <t>free-white age-band fingerprint over 26 of the schedule's 26 columns matches exactly one of the 964 IPUMS households</t>
+        </is>
+      </c>
+      <c r="O684" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B685" t="n">
+        <v>212</v>
+      </c>
+      <c r="C685" t="n">
+        <v>18</v>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>F[r]. Ka[l]bfl[ei]sch</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>[?] Kalbfleisch</t>
+        </is>
+      </c>
+      <c r="F685" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G685" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H685" t="inlineStr">
+        <is>
+          <t>5101405</t>
+        </is>
+      </c>
+      <c r="I685" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
+      <c r="J685" t="n">
+        <v>26</v>
+      </c>
+      <c r="K685" t="inlineStr"/>
+      <c r="L685" t="inlineStr"/>
+      <c r="M685" t="inlineStr"/>
+      <c r="N685" t="inlineStr">
+        <is>
+          <t>free-white age-band fingerprint over 26 of the schedule's 26 columns matches exactly one of the 964 IPUMS households</t>
+        </is>
+      </c>
+      <c r="O685" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B686" t="n">
+        <v>212</v>
+      </c>
+      <c r="C686" t="n">
+        <v>19</v>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>Jam[e]s [?] Morrison</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>James Morrison</t>
+        </is>
+      </c>
+      <c r="F686" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G686" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H686" t="inlineStr"/>
+      <c r="I686" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J686" t="n">
+        <v>26</v>
+      </c>
+      <c r="K686" t="inlineStr"/>
+      <c r="L686" t="inlineStr"/>
+      <c r="M686" t="inlineStr"/>
+      <c r="N686" t="inlineStr">
+        <is>
+          <t>no IPUMS household carries this pattern over the 26 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
+        </is>
+      </c>
+      <c r="O686" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B687" t="n">
+        <v>212</v>
+      </c>
+      <c r="C687" t="n">
+        <v>20</v>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>L. Chr[is]t[ia]n[s]</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>L. Christians</t>
+        </is>
+      </c>
+      <c r="F687" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G687" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H687" t="inlineStr"/>
+      <c r="I687" t="inlineStr">
+        <is>
+          <t>ambiguous(4)</t>
+        </is>
+      </c>
+      <c r="J687" t="n">
+        <v>26</v>
+      </c>
+      <c r="K687" t="inlineStr">
+        <is>
+          <t>5101377;5101407;5101520;5101592</t>
+        </is>
+      </c>
+      <c r="L687" t="inlineStr">
+        <is>
+          <t>5101407</t>
+        </is>
+      </c>
+      <c r="M687" t="inlineStr">
+        <is>
+          <t>lines 18 and 23 resolve uniquely to serials 5101405 and 5101410; of this line's 4 candidates exactly one, 5101407, lies in that run at exactly the position an unbroken run would put it</t>
+        </is>
+      </c>
+      <c r="N687" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 4 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O687" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B688" t="n">
+        <v>212</v>
+      </c>
+      <c r="C688" t="n">
+        <v>21</v>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>Geo. C. Mo[r]e</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>George C. More</t>
+        </is>
+      </c>
+      <c r="F688" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G688" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H688" t="inlineStr"/>
+      <c r="I688" t="inlineStr">
+        <is>
+          <t>ambiguous(3)</t>
+        </is>
+      </c>
+      <c r="J688" t="n">
+        <v>26</v>
+      </c>
+      <c r="K688" t="inlineStr">
+        <is>
+          <t>5101408;5101409;5101459</t>
+        </is>
+      </c>
+      <c r="L688" t="inlineStr"/>
+      <c r="M688" t="inlineStr">
+        <is>
+          <t>lines 18 and 23 resolve uniquely to serials 5101405 and 5101410, and 2 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
+        </is>
+      </c>
+      <c r="N688" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 3 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O688" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B689" t="n">
+        <v>212</v>
+      </c>
+      <c r="C689" t="n">
+        <v>22</v>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>[J]. Kir[t]la[n]d</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>J. Kirtland</t>
+        </is>
+      </c>
+      <c r="F689" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G689" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H689" t="inlineStr"/>
+      <c r="I689" t="inlineStr">
+        <is>
+          <t>ambiguous(3)</t>
+        </is>
+      </c>
+      <c r="J689" t="n">
+        <v>26</v>
+      </c>
+      <c r="K689" t="inlineStr">
+        <is>
+          <t>5101408;5101409;5101459</t>
+        </is>
+      </c>
+      <c r="L689" t="inlineStr"/>
+      <c r="M689" t="inlineStr">
+        <is>
+          <t>lines 18 and 23 resolve uniquely to serials 5101405 and 5101410, and 2 of this line's candidates fall between them, so continuity narrows and does not settle it</t>
+        </is>
+      </c>
+      <c r="N689" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 3 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O689" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B690" t="n">
+        <v>212</v>
+      </c>
+      <c r="C690" t="n">
+        <v>23</v>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>Jas. Edmu[n]ds</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>James Edmunds</t>
+        </is>
+      </c>
+      <c r="F690" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G690" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H690" t="inlineStr">
+        <is>
+          <t>5101410</t>
+        </is>
+      </c>
+      <c r="I690" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
+      <c r="J690" t="n">
+        <v>26</v>
+      </c>
+      <c r="K690" t="inlineStr"/>
+      <c r="L690" t="inlineStr"/>
+      <c r="M690" t="inlineStr"/>
+      <c r="N690" t="inlineStr">
+        <is>
+          <t>free-white age-band fingerprint over 26 of the schedule's 26 columns matches exactly one of the 964 IPUMS households</t>
+        </is>
+      </c>
+      <c r="O690" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B691" t="n">
+        <v>212</v>
+      </c>
+      <c r="C691" t="n">
+        <v>24</v>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>John P[e]irc[e]</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>John Peirce</t>
+        </is>
+      </c>
+      <c r="F691" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G691" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H691" t="inlineStr"/>
+      <c r="I691" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J691" t="n">
+        <v>26</v>
+      </c>
+      <c r="K691" t="inlineStr"/>
+      <c r="L691" t="inlineStr"/>
+      <c r="M691" t="inlineStr"/>
+      <c r="N691" t="inlineStr">
+        <is>
+          <t>no IPUMS household carries this pattern over the 26 compared columns — either the household is outside the extract or the reading of one cell is wrong, and this tool cannot tell those apart</t>
+        </is>
+      </c>
+      <c r="O691" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B692" t="n">
+        <v>212</v>
+      </c>
+      <c r="C692" t="n">
+        <v>25</v>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>[P]. Lawrence</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>P. Lawrence</t>
+        </is>
+      </c>
+      <c r="F692" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G692" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H692" t="inlineStr">
+        <is>
+          <t>5101412</t>
+        </is>
+      </c>
+      <c r="I692" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
+      <c r="J692" t="n">
+        <v>26</v>
+      </c>
+      <c r="K692" t="inlineStr"/>
+      <c r="L692" t="inlineStr"/>
+      <c r="M692" t="inlineStr"/>
+      <c r="N692" t="inlineStr">
+        <is>
+          <t>free-white age-band fingerprint over 26 of the schedule's 26 columns matches exactly one of the 964 IPUMS households</t>
+        </is>
+      </c>
+      <c r="O692" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B693" t="n">
+        <v>212</v>
+      </c>
+      <c r="C693" t="n">
+        <v>26</v>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>[J]. [C]. Walker</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>J. C. Walker</t>
+        </is>
+      </c>
+      <c r="F693" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G693" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H693" t="inlineStr"/>
+      <c r="I693" t="inlineStr">
+        <is>
+          <t>ambiguous(10)</t>
+        </is>
+      </c>
+      <c r="J693" t="n">
+        <v>26</v>
+      </c>
+      <c r="K693" t="inlineStr">
+        <is>
+          <t>5101381;5101393;5101398;5101413;5101423;5101446;5101456;5101594;5101595;5101596</t>
+        </is>
+      </c>
+      <c r="L693" t="inlineStr">
+        <is>
+          <t>5101413</t>
+        </is>
+      </c>
+      <c r="M693" t="inlineStr">
+        <is>
+          <t>lines 25 and 27 resolve uniquely to serials 5101412 and 5101414; of this line's 10 candidates exactly one, 5101413, lies in that run at exactly the position an unbroken run would put it</t>
+        </is>
+      </c>
+      <c r="N693" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 10 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O693" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B694" t="n">
+        <v>212</v>
+      </c>
+      <c r="C694" t="n">
+        <v>27</v>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>[W]m. Williams</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>William Williams</t>
+        </is>
+      </c>
+      <c r="F694" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G694" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H694" t="inlineStr">
+        <is>
+          <t>5101414</t>
+        </is>
+      </c>
+      <c r="I694" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
+      <c r="J694" t="n">
+        <v>26</v>
+      </c>
+      <c r="K694" t="inlineStr"/>
+      <c r="L694" t="inlineStr"/>
+      <c r="M694" t="inlineStr"/>
+      <c r="N694" t="inlineStr">
+        <is>
+          <t>free-white age-band fingerprint over 26 of the schedule's 26 columns matches exactly one of the 964 IPUMS households</t>
+        </is>
+      </c>
+      <c r="O694" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B695" t="n">
+        <v>212</v>
+      </c>
+      <c r="C695" t="n">
+        <v>28</v>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>W. Nelson</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>W. Nelson</t>
+        </is>
+      </c>
+      <c r="F695" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G695" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H695" t="inlineStr">
+        <is>
+          <t>5101415</t>
+        </is>
+      </c>
+      <c r="I695" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
+      <c r="J695" t="n">
+        <v>26</v>
+      </c>
+      <c r="K695" t="inlineStr"/>
+      <c r="L695" t="inlineStr"/>
+      <c r="M695" t="inlineStr"/>
+      <c r="N695" t="inlineStr">
+        <is>
+          <t>free-white age-band fingerprint over 26 of the schedule's 26 columns matches exactly one of the 964 IPUMS households</t>
+        </is>
+      </c>
+      <c r="O695" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B696" t="n">
+        <v>212</v>
+      </c>
+      <c r="C696" t="n">
+        <v>29</v>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>Geo. Merrill</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>George Merrill</t>
+        </is>
+      </c>
+      <c r="F696" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G696" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H696" t="inlineStr"/>
+      <c r="I696" t="inlineStr">
+        <is>
+          <t>ambiguous(6)</t>
+        </is>
+      </c>
+      <c r="J696" t="n">
+        <v>26</v>
+      </c>
+      <c r="K696" t="inlineStr">
+        <is>
+          <t>5101417;5101455;5101610;5102008;5102024;5102179</t>
+        </is>
+      </c>
+      <c r="L696" t="inlineStr"/>
+      <c r="M696" t="inlineStr"/>
+      <c r="N696" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 6 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O696" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B697" t="n">
+        <v>212</v>
+      </c>
+      <c r="C697" t="n">
+        <v>30</v>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>J. W. Salisbury</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>J. W. Salisbury</t>
+        </is>
+      </c>
+      <c r="F697" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G697" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H697" t="inlineStr"/>
+      <c r="I697" t="inlineStr">
+        <is>
+          <t>ambiguous(10)</t>
+        </is>
+      </c>
+      <c r="J697" t="n">
+        <v>26</v>
+      </c>
+      <c r="K697" t="inlineStr">
+        <is>
+          <t>5101266;5101418;5101462;5101512;5101640;5101645;5101664;5101751;5101960;5102190</t>
+        </is>
+      </c>
+      <c r="L697" t="inlineStr"/>
+      <c r="M697" t="inlineStr"/>
+      <c r="N697" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 10 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O697" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>33SQ-GYYJ-RY</t>
+        </is>
+      </c>
+      <c r="B698" t="n">
+        <v>212</v>
+      </c>
+      <c r="C698" t="n">
+        <v>31</v>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>John Parkin</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>John Parkin</t>
+        </is>
+      </c>
+      <c r="F698" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G698" t="inlineStr">
+        <is>
+          <t>scan_verified</t>
+        </is>
+      </c>
+      <c r="H698" t="inlineStr"/>
+      <c r="I698" t="inlineStr">
+        <is>
+          <t>ambiguous(43)</t>
+        </is>
+      </c>
+      <c r="J698" t="n">
+        <v>26</v>
+      </c>
+      <c r="K698" t="inlineStr">
+        <is>
+          <t>5101373;5101374;5101375;5101376;5101378;5101401;5101402;5101403;5101406;5101419;5101421;5101433;5101454;5101458;5101460;5101469;5101494;5101499;5101500;5101501;5101508;5101511;5101513;5101518;5101523;5101524;5101558;5101587;5101590;5101598;5101600;5101612;5101613;5101622;5101623;5101633;5101637;5101646;5101676;5101746;5102034;5102173;5102174</t>
+        </is>
+      </c>
+      <c r="L698" t="inlineStr"/>
+      <c r="M698" t="inlineStr"/>
+      <c r="N698" t="inlineStr">
+        <is>
+          <t>the fingerprint over 26 columns matches 43 IPUMS households and does not distinguish them; no serial is attached</t>
+        </is>
+      </c>
+      <c r="O698" t="inlineStr">
+        <is>
+          <t>chicago/reference/census1840/33SQ-GYYJ-RY.jpg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>